<commit_message>
更新 2026-08-17 風險新聞明細（2026-08-17 14:23）
</commit_message>
<xml_diff>
--- a/risk_news_daily/2026-08-17.xlsx
+++ b/risk_news_daily/2026-08-17.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="風險新聞" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'風險新聞'!$A$1:$O$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'風險新聞'!$A$1:$O$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O101"/>
+  <dimension ref="A1:O100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -533,12 +533,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Walmart</t>
+          <t>Intercontinental Exchange</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -604,12 +604,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Intercontinental Exchange</t>
+          <t>Walmart</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1309,45 +1309,45 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 05:45:00</t>
+          <t>2026-08-17 05:24:00</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>TSCO</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Realty Income</t>
+          <t>Tractor Supply</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Celtic Keeping Close Tabs On This Swedish Goalkeeper: Should O’Neill Sanction The Move?</t>
+          <t>California settlement hits Tractor Supply over pricing, pesticides, and 'biodegradable' claims</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>凱爾特人密切關注這位瑞典門將：奧尼爾應該批准這一舉動嗎？</t>
+          <t>加州和解協議對拖拉機供應公司的定價、殺蟲劑和「可生物降解」索賠造成打擊</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-0.133</v>
+        <v>-0.952</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>GEOPOLITICAL</t>
+          <t>LEGAL</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>SANCTION</t>
+          <t>REGULATORY_PENALTY</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>制裁</t>
+          <t>監管裁罰</t>
         </is>
       </c>
       <c r="J13" s="2" t="n">
@@ -1360,17 +1360,17 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>sanction</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOS1ZHaGxIS3J6RFFJeExwVmNOcTQxcHpmVFlIV09OMjVDN2dfWVRvbUhMYnp0bUhHMkRhZ0M0UHpSZG40T081QUcxREw2LTdwNnd1TzB0VG5pTVJzaHNrbW0yQmR6UlQ5LUw4cHNua3lxNE9QbmcxUUt2cWg1TUo3VDRyZnhKRWpfSkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQaThaYWFOUUdFS0VKSU5Jc0NMVUx6ekFXRk0zQzlrSExRc0RWbUhfQzEzNEFaRnluXzJma2ZfSi1McEpqb29Ib0VSMDlzMkFmVlJPbVhWZ2ctRjVGQnAtZ25DREhGYWxDZ3VhVk9icnN3dmpBRW9ZbVhDRnJvblVGeUg0M2pEVXI4dkJxM2o2Q1BOc2ptY0xrLTh0LUp3dUpmVGZDTk9jQm9lVXk4ZEkxbWsta3VLYTQzeFE?oc=5</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports</t>
+          <t>The Cool Down</t>
         </is>
       </c>
       <c r="O13" s="2" t="b">
@@ -1380,31 +1380,31 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 05:24:00</t>
+          <t>2026-08-17 05:06:39</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>TSCO</t>
+          <t>COF</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Tractor Supply</t>
+          <t>Capital One</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>California settlement hits Tractor Supply over pricing, pesticides, and 'biodegradable' claims</t>
+          <t>Boy George - Radio Interview (3 Jul 26) Capital One Class Action Lawsuit (61jGcnyHu9)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>加州和解協議對拖拉機供應公司的定價、殺蟲劑和「可生物降解」索賠造成打擊</t>
+          <t>Boy George - 電台訪談（26 年 7 月 3 日）第一資本集體訴訟 (61jGcnyHu9)</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-0.952</v>
+        <v>-0.232</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -1413,12 +1413,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>REGULATORY_PENALTY</t>
+          <t>MAJOR_LITIGATION</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>監管裁罰</t>
+          <t>重大訴訟</t>
         </is>
       </c>
       <c r="J14" s="2" t="n">
@@ -1431,17 +1431,17 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>class action</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQaThaYWFOUUdFS0VKSU5Jc0NMVUx6ekFXRk0zQzlrSExRc0RWbUhfQzEzNEFaRnluXzJma2ZfSi1McEpqb29Ib0VSMDlzMkFmVlJPbVhWZ2ctRjVGQnAtZ25DREhGYWxDZ3VhVk9icnN3dmpBRW9ZbVhDRnJvblVGeUg0M2pEVXI4dkJxM2o2Q1BOc2ptY0xrLTh0LUp3dUpmVGZDTk9jQm9lVXk4ZEkxbWsta3VLYTQzeFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFBsZlRfNXdiVjV3OTFrMGNxM2JOcmVOY2tWQloxeXJuZWJhenJmblc0VC1sOTRkZWxIeEhfNjR0T2tvTmJYLVJDd29HbWczMVkzNWZkUTNjQ2dBTHM?oc=5</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>The Cool Down</t>
+          <t>Mshale</t>
         </is>
       </c>
       <c r="O14" s="2" t="b">
@@ -1451,31 +1451,31 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 05:06:39</t>
+          <t>2026-08-17 02:31:00</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>COF</t>
+          <t>PODD</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Capital One</t>
+          <t>Insulet Corporation</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Boy George - Radio Interview (3 Jul 26) Capital One Class Action Lawsuit (61jGcnyHu9)</t>
+          <t>PODD UPCOMING DEADLINE: Faruqi &amp; Faruqi, LLP Reminds Insulet (PODD) Investors of Securities Class Action Lawsuit Deadline on August 31, 2026</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Boy George - 電台訪談（26 年 7 月 3 日）第一資本集體訴訟 (61jGcnyHu9)</t>
+          <t>PODD 截止日期即將到來：Faruqi &amp; Faruqi, LLP 提醒 Insulet (PODD) 投資者證券集體訴訟截止日期為 2026 年 8 月 31 日</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-0.232</v>
+        <v>-0.065</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
@@ -1507,12 +1507,12 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFBsZlRfNXdiVjV3OTFrMGNxM2JOcmVOY2tWQloxeXJuZWJhenJmblc0VC1sOTRkZWxIeEhfNjR0T2tvTmJYLVJDd29HbWczMVkzNWZkUTNjQ2dBTHM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAJBVV95cUxNZlJ3S0xCR2RwRHY1djNQNnYyX29Vd1YwUXhoNGkzWG1vRkxtck9Oamx3WEFCQUZiQVJWbnZBNFJYTm9fRklCVUpnQTVFb1ZQVVI2QW5sdnVlUmJ2NkdIZHRNc242alowMjFMdDA5ejd6eVZpRDB6X3NBTnpISU1FSUZkWlgyVmc1Y1JZbFFwckFwLTVQbmVTZHpocjZuWkpKaV84elp6R2ZCRXZtcjAxcjMzaVNhREpubldSV0FEVVFCQTJnQWl3N3RiejU5Rlc5bTF4OGdCSTFvaUpSQkRNQW1tam8tX2ZWVURiNkViYVBfUGhMM05oU2RfamdHTjRqSllzUnBPak8?oc=5</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Mshale</t>
+          <t>TMX Newsfile</t>
         </is>
       </c>
       <c r="O15" s="2" t="b">
@@ -1522,31 +1522,31 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 02:31:00</t>
+          <t>2026-08-17 01:00:00</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>PODD</t>
+          <t>PNR</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Insulet Corporation</t>
+          <t>Pentair</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>PODD UPCOMING DEADLINE: Faruqi &amp; Faruqi, LLP Reminds Insulet (PODD) Investors of Securities Class Action Lawsuit Deadline on August 31, 2026</t>
+          <t>2026-08-16 | PNR STOCKHOLDER ALERT: Bronstein, Gewirtz and Grossman, LLC Announces that Pentair plc Investors with Substantial Losses Have Opportunity to Lead Class Action Lawsuit! | NYSE:PNR | Press Release</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>PODD 截止日期即將到來：Faruqi &amp; Faruqi, LLP 提醒 Insulet (PODD) 投資者證券集體訴訟截止日期為 2026 年 8 月 31 日</t>
+          <t>2026-08-16 | PNR 股東提醒：Bronstein、Gewirtz 和 Grossman, LLC 宣布遭受重大損失的 Pentair plc 投資者有機會提起集體訴訟！ |紐約證券交易所：PNR |新聞稿</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-0.065</v>
+        <v>-0.7</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
@@ -1578,12 +1578,12 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAJBVV95cUxNZlJ3S0xCR2RwRHY1djNQNnYyX29Vd1YwUXhoNGkzWG1vRkxtck9Oamx3WEFCQUZiQVJWbnZBNFJYTm9fRklCVUpnQTVFb1ZQVVI2QW5sdnVlUmJ2NkdIZHRNc242alowMjFMdDA5ejd6eVZpRDB6X3NBTnpISU1FSUZkWlgyVmc1Y1JZbFFwckFwLTVQbmVTZHpocjZuWkpKaV84elp6R2ZCRXZtcjAxcjMzaVNhREpubldSV0FEVVFCQTJnQWl3N3RiejU5Rlc5bTF4OGdCSTFvaUpSQkRNQW1tam8tX2ZWVURiNkViYVBfUGhMM05oU2RfamdHTjRqSllzUnBPak8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOQ1kybWpYemNLWEFXdm9Fc1hnR0pOWkNqWkluSWJFMWtkRmNKMDJLRUs1dk5OeEdWSGY3LUZFUVU1cms2dkJaODZDVTdXQmlWTkxQcFcxTVJtVURVbk5zMUhWdkJaeEFIcFRNcjRQUzl5dWJnTDdjWXdFdWlmWF9pTkJvNngwVVhxUE8xMnlMMnJPUFdWMkVSMWpZaVlRWXppdnNnSVBIcnFJN1F4eFFvcGpfWGtZQ0ptOGdXY3N0VmJ4dFdWX3hFZTNCcjRaUQ?oc=5</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>TMX Newsfile</t>
+          <t>Stockhouse</t>
         </is>
       </c>
       <c r="O16" s="2" t="b">
@@ -1593,31 +1593,31 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 01:00:00</t>
+          <t>2026-08-17 00:00:00</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PNR</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Pentair</t>
+          <t>Regeneron Pharmaceuticals</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 | PNR STOCKHOLDER ALERT: Bronstein, Gewirtz and Grossman, LLC Announces that Pentair plc Investors with Substantial Losses Have Opportunity to Lead Class Action Lawsuit! | NYSE:PNR | Press Release</t>
+          <t>Bronstein, Gewirtz &amp; Grossman LLC Urges Regeneron Pharmaceuticals, Inc. Investors to Act: Class Action Filed Alleging Investor Harm</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 | PNR 股東提醒：Bronstein、Gewirtz 和 Grossman, LLC 宣布遭受重大損失的 Pentair plc 投資者有機會提起集體訴訟！ |紐約證券交易所：PNR |新聞稿</t>
+          <t>Bronstein, Gewirtz &amp; Grossman LLC 敦促 Regeneron Pharmaceuticals, Inc. 投資者採取行動：提起集體訴訟，指控投資者受到傷害</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>-0.7</v>
+        <v>-0.611</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -1649,12 +1649,12 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOQ1kybWpYemNLWEFXdm9Fc1hnR0pOWkNqWkluSWJFMWtkRmNKMDJLRUs1dk5OeEdWSGY3LUZFUVU1cms2dkJaODZDVTdXQmlWTkxQcFcxTVJtVURVbk5zMUhWdkJaeEFIcFRNcjRQUzl5dWJnTDdjWXdFdWlmWF9pTkJvNngwVVhxUE8xMnlMMnJPUFdWMkVSMWpZaVlRWXppdnNnSVBIcnFJN1F4eFFvcGpfWGtZQ0ptOGdXY3N0VmJ4dFdWX3hFZTNCcjRaUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwJBVV95cUxNQlFEaVkySW9lWldHTWR0aXdTaVlOeC0xRFpMVjRSUWxlbHNUWXhULUFUTFVEcTVkQnpsN1pSTW4xSjB6ZlNJZGczTlQzcnhWbjBhMXRiZEFaZXIyMkg1M2dISFBfM1NJTC1mQzA0dVFKRmk2ektJR1VnZGczdlFMbG1BYkt2WUZlNXBSdm8xUFM1WlBGdzM3NHoxZV9XZGItNmthdkJoc2xoa19PMmRXSV9LOUZ1dE1mVzhXVHdIOG8zMlowNm81dGc2SjF3cTlHUnlpRE9kdFNPLTgyTzdRZ0QzT2pWc2lSSDRldTJKZEpObWZuMm04U0Uxb3R5bXgxQTM5cUN1M3lJZ3g5SFdKMFI5bEY1dEg3SWgzNmVXV1BSUjhBczZrSWk4Ul9oMGhFbEJGWFZpSFZ2Ymc?oc=5</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Stockhouse</t>
+          <t>mykxlg.com</t>
         </is>
       </c>
       <c r="O17" s="2" t="b">
@@ -1664,31 +1664,31 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 00:00:00</t>
+          <t>2026-08-16 21:31:48</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Regeneron Pharmaceuticals</t>
+          <t>Kroger</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Bronstein, Gewirtz &amp; Grossman LLC Urges Regeneron Pharmaceuticals, Inc. Investors to Act: Class Action Filed Alleging Investor Harm</t>
+          <t>Every Super League club’s penalty points with Hull KR most ill-disciplined</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Bronstein, Gewirtz &amp; Grossman LLC 敦促 Regeneron Pharmaceuticals, Inc. 投資者採取行動：提起集體訴訟，指控投資者受到傷害</t>
+          <t>各中超俱樂部罰分最多，赫爾KR紀律最差</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>-0.611</v>
+        <v>-0.894</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1697,12 +1697,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>MAJOR_LITIGATION</t>
+          <t>REGULATORY_PENALTY</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>重大訴訟</t>
+          <t>監管裁罰</t>
         </is>
       </c>
       <c r="J18" s="2" t="n">
@@ -1715,17 +1715,17 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>class action</t>
+          <t>penalty</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwJBVV95cUxNQlFEaVkySW9lWldHTWR0aXdTaVlOeC0xRFpMVjRSUWxlbHNUWXhULUFUTFVEcTVkQnpsN1pSTW4xSjB6ZlNJZGczTlQzcnhWbjBhMXRiZEFaZXIyMkg1M2dISFBfM1NJTC1mQzA0dVFKRmk2ektJR1VnZGczdlFMbG1BYkt2WUZlNXBSdm8xUFM1WlBGdzM3NHoxZV9XZGItNmthdkJoc2xoa19PMmRXSV9LOUZ1dE1mVzhXVHdIOG8zMlowNm81dGc2SjF3cTlHUnlpRE9kdFNPLTgyTzdRZ0QzT2pWc2lSSDRldTJKZEpObWZuMm04U0Uxb3R5bXgxQTM5cUN1M3lJZ3g5SFdKMFI5bEY1dEg3SWgzNmVXV1BSUjhBczZrSWk4Ul9oMGhFbEJGWFZpSFZ2Ymc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOVUlCV2VjTVpGUGh0NXY2X3VON1A0UGVoLWFCYTljSU1WMEJXM2VDMzByekM1ZUd2dmQ5ZEw5cE8wckhOdElvZ1RvRmcydVhRNkhoM0VDOFQxTWRtYk5GSHRKekp1QnBNcFBPSGNlWGlyUUNnRDF1QVZNMDBFSlJOT3dTVnNUZHBtWHRubjdNQjV1aGJ1clgyLXJEazFTRl84ei1helZmS0lwWlNZaUpuSUtuVWVxbHpMbEhwbHNwZTVCekdibmZXODhR0gHPAUFVX3lxTFBuSG1Mc2lYQXYtbWVCeU9jQkp1WW5pUUpEcUwwalVtNGZROFl1QTVJMnk3OHdBYlY1SGRwMmwxWDkyVWxqbzRJMEg5emZGNEVJLWRtOXlxa0JLMEZVLS1INk1CSm1Ib0JzR05rRTFjZGZCMFlJRmRqZ1RyeWotY1plYVJCcDMzdVJ2bU9GVmtmdTk5S0tuSzYxWnIwSHh4YndCaFhKb01fLXk0a0poZUdtVXpWUkwxbHAyQ3kzVV9tYW40c1V3WDR4VmRQbElsUQ?oc=5</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>mykxlg.com</t>
+          <t>Serious About Rugby League</t>
         </is>
       </c>
       <c r="O18" s="2" t="b">
@@ -1735,31 +1735,31 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 21:31:48</t>
+          <t>2026-08-16 21:20:03</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>HUM</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Kroger</t>
+          <t>Humana</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Every Super League club’s penalty points with Hull KR most ill-disciplined</t>
+          <t>Federal Judge Approves $3 Million Settlement In Willows Apartments Class-action Lawsuit Humana (LBYlYVW19j)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>各中超俱樂部罰分最多，赫爾KR紀律最差</t>
+          <t>聯邦法官批准 Willows Apartments 集體訴訟 Humana 獲得 300 萬美元和解 (LBYlYVW19j)</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>-0.894</v>
+        <v>0.494</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
@@ -1786,17 +1786,17 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>penalty</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOVUlCV2VjTVpGUGh0NXY2X3VON1A0UGVoLWFCYTljSU1WMEJXM2VDMzByekM1ZUd2dmQ5ZEw5cE8wckhOdElvZ1RvRmcydVhRNkhoM0VDOFQxTWRtYk5GSHRKekp1QnBNcFBPSGNlWGlyUUNnRDF1QVZNMDBFSlJOT3dTVnNUZHBtWHRubjdNQjV1aGJ1clgyLXJEazFTRl84ei1helZmS0lwWlNZaUpuSUtuVWVxbHpMbEhwbHNwZTVCekdibmZXODhR0gHPAUFVX3lxTFBuSG1Mc2lYQXYtbWVCeU9jQkp1WW5pUUpEcUwwalVtNGZROFl1QTVJMnk3OHdBYlY1SGRwMmwxWDkyVWxqbzRJMEg5emZGNEVJLWRtOXlxa0JLMEZVLS1INk1CSm1Ib0JzR05rRTFjZGZCMFlJRmRqZ1RyeWotY1plYVJCcDMzdVJ2bU9GVmtmdTk5S0tuSzYxWnIwSHh4YndCaFhKb01fLXk0a0poZUdtVXpWUkwxbHAyQ3kzVV9tYW40c1V3WDR4VmRQbElsUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTE9CampqMkl6dkpTaW1PeV9PUjZ0TU54VG1lbmVGLVczMzI0UDJRamFVU01kR0NFLVl4WVFhS3ZlN0ZnSE0teXdpRVRJdXo4SllkLS1xeVdrNGlXWWZVN1hfNQ?oc=5</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Serious About Rugby League</t>
+          <t>Mshale</t>
         </is>
       </c>
       <c r="O19" s="2" t="b">
@@ -1806,31 +1806,31 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 21:20:03</t>
+          <t>2026-08-16 21:06:01</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>HUM</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Humana</t>
+          <t>AppLovin</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Federal Judge Approves $3 Million Settlement In Willows Apartments Class-action Lawsuit Humana (LBYlYVW19j)</t>
+          <t>Apple class action alleges App Store failed to stop fake crypto wallet app</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>聯邦法官批准 Willows Apartments 集體訴訟 Humana 獲得 300 萬美元和解 (LBYlYVW19j)</t>
+          <t>蘋果集體訴訟稱 App Store 未能阻止假加密錢包應用</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.494</v>
+        <v>-0.824</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -1839,12 +1839,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>REGULATORY_PENALTY</t>
+          <t>MAJOR_LITIGATION</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>監管裁罰</t>
+          <t>重大訴訟</t>
         </is>
       </c>
       <c r="J20" s="2" t="n">
@@ -1857,17 +1857,17 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>class action</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTE9CampqMkl6dkpTaW1PeV9PUjZ0TU54VG1lbmVGLVczMzI0UDJRamFVU01kR0NFLVl4WVFhS3ZlN0ZnSE0teXdpRVRJdXo4SllkLS1xeVdrNGlXWWZVN1hfNQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQY3V1aFc4ZjFwZUlmQWJiV3hMZTI3SUFMVDJkdXBCU0tjbjVTdXlENU51SmFwSnhMZW1Ha0hzNDNkM2hnMEN4SGl1WWtSd01Ma0hJeUR0SEV1SFlFRC1sRjhqc3dNaXkxa2VkcTBwZE81bDVCYVZRd0tYdGxQNi1PM0J5MXBsWU54QWg0dkJEbTIxbWV2eElzYWFxeE1WcFhoRWhyVmx4OGVNVFl5UXRaeFo3RVU4SWEyN3hWSFg4VWl0VHRYUUx3MWNQTUJMTVJSY0E?oc=5</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Mshale</t>
+          <t>Top Class Actions</t>
         </is>
       </c>
       <c r="O20" s="2" t="b">
@@ -1877,31 +1877,31 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 21:06:01</t>
+          <t>2026-08-16 21:05:09</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>AppLovin</t>
+          <t>Cencora</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Apple class action alleges App Store failed to stop fake crypto wallet app</t>
+          <t>FRONTAL TRUST ADM COR REND CON LIQUIDE CLPP Balance Sheet – BCS:CFIFTCLP_E1</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>蘋果集體訴訟稱 App Store 未能阻止假加密錢包應用</t>
+          <t>FRONTAL TRUST ADM COR REND CON LIQUIDE CLPP 資產負債表 – BCS:CFIFTCLP_E1</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>-0.824</v>
+        <v>0.019</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -1910,12 +1910,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>MAJOR_LITIGATION</t>
+          <t>REGULATORY_INVESTIGATION</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>重大訴訟</t>
+          <t>監管調查</t>
         </is>
       </c>
       <c r="J21" s="2" t="n">
@@ -1928,17 +1928,17 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>class action</t>
+          <t>FTC</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQY3V1aFc4ZjFwZUlmQWJiV3hMZTI3SUFMVDJkdXBCU0tjbjVTdXlENU51SmFwSnhMZW1Ha0hzNDNkM2hnMEN4SGl1WWtSd01Ma0hJeUR0SEV1SFlFRC1sRjhqc3dNaXkxa2VkcTBwZE81bDVCYVZRd0tYdGxQNi1PM0J5MXBsWU54QWg0dkJEbTIxbWV2eElzYWFxeE1WcFhoRWhyVmx4OGVNVFl5UXRaeFo3RVU4SWEyN3hWSFg4VWl0VHRYUUx3MWNQTUJMTVJSY0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNZjlzb3hZUDZ5dnFPTHppR3hOS0dtc3haUGJVRVM5eUFfN1dYenlCNkZIcHR5azl3eHdqTUs4SDI3dFRnYUJfSU10Yjd4c1FmNHprNWJ0N3dGZngxd3lhQ0paMko5X25tMWllcjlKX3VoX25hODVfUm9uRE5kSC1iNkN3RQ?oc=5</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>Top Class Actions</t>
+          <t>TradingView</t>
         </is>
       </c>
       <c r="O21" s="2" t="b">
@@ -1953,12 +1953,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>ADM</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Cencora</t>
+          <t>Archer Daniels Midland</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2019,45 +2019,45 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 21:05:09</t>
+          <t>2026-08-16 20:38:00</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>ADM</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Archer Daniels Midland</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>FRONTAL TRUST ADM COR REND CON LIQUIDE CLPP Balance Sheet – BCS:CFIFTCLP_E1</t>
+          <t>Bristol private hire driver stripped of licence after Uber sexual misconduct reports</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>FRONTAL TRUST ADM COR REND CON LIQUIDE CLPP 資產負債表 – BCS:CFIFTCLP_E1</t>
+          <t>布里斯托爾私人僱傭司機因 Uber 不當性行為報告被吊銷駕照</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0.019</v>
+        <v>-0.827</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>LEGAL</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>REGULATORY_INVESTIGATION</t>
+          <t>EXECUTIVE_MISCONDUCT</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>監管調查</t>
+          <t>高管不當行為</t>
         </is>
       </c>
       <c r="J23" s="2" t="n">
@@ -2070,17 +2070,17 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>FTC</t>
+          <t>misconduct</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNZjlzb3hZUDZ5dnFPTHppR3hOS0dtc3haUGJVRVM5eUFfN1dYenlCNkZIcHR5azl3eHdqTUs4SDI3dFRnYUJfSU10Yjd4c1FmNHprNWJ0N3dGZngxd3lhQ0paMko5X25tMWllcjlKX3VoX25hODVfUm9uRE5kSC1iNkN3RQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPQ2tzUUJZMXZCdVlNS1dzaXZHVGVBS1dkOEs1UktUMzNTX1VuQ0J0ZV9zUWFyWW5VQkVYeFhsNjhSNHFsbi1DYnlZQ3h1TWlmSU9RajVnaHJJanBRUDVGVXpQNllPcmR0ZEtrWHg4YVlzempHZWRWQjZtdFNpSWNxZGx6NngwcE9DNE5taTYyQTg1YU00ZDZDcnY3X1FzOUJiV2tFQzdfbXNGTHBLaG00cERScW8xR3AyRWc?oc=5</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>TradingView</t>
+          <t>taxi-point.co.uk</t>
         </is>
       </c>
       <c r="O23" s="2" t="b">
@@ -2090,45 +2090,45 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 20:38:00</t>
+          <t>2026-08-16 19:38:27</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>FSLR</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>First Solar</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Bristol private hire driver stripped of licence after Uber sexual misconduct reports</t>
+          <t>FSLR Stockholders Have Opportunity to Lead First Solar, Inc. Class Action Lawsuit – Contact Bronstein, Gewirtz and Grossman, LLC Today!</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>布里斯托爾私人僱傭司機因 Uber 不當性行為報告被吊銷駕照</t>
+          <t>FSLR 股東有機會領導 First Solar, Inc. 集體訴訟 – 立即聯繫 Bronstein、Gewirtz 和 Grossman, LLC！</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>-0.827</v>
+        <v>0.053</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>GOVERNANCE</t>
+          <t>LEGAL</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>EXECUTIVE_MISCONDUCT</t>
+          <t>MAJOR_LITIGATION</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>高管不當行為</t>
+          <t>重大訴訟</t>
         </is>
       </c>
       <c r="J24" s="2" t="n">
@@ -2141,17 +2141,17 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>misconduct</t>
+          <t>class action</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPQ2tzUUJZMXZCdVlNS1dzaXZHVGVBS1dkOEs1UktUMzNTX1VuQ0J0ZV9zUWFyWW5VQkVYeFhsNjhSNHFsbi1DYnlZQ3h1TWlmSU9RajVnaHJJanBRUDVGVXpQNllPcmR0ZEtrWHg4YVlzempHZWRWQjZtdFNpSWNxZGx6NngwcE9DNE5taTYyQTg1YU00ZDZDcnY3X1FzOUJiV2tFQzdfbXNGTHBLaG00cERScW8xR3AyRWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPYTRpVkpjZkxxY0JlcS1TeUVvaGRDRzUtMzFDMFFGRUZkYjNQMWFLOUVjdjFlNUdsMUNsRE5ZSWhUTHJYcEdNQmxuUFM4TC1PNENMTUQ1WVJDTk9YcmlGY0szRThtdHM3ZXFUVy1BcGhfQnB1RW1zNWtDTHk4ek94MzZ3bzBFbkdZZHFZZzNjMXI4b2FsQXpEUkktMF9iTUVwSWVSMEducmExRGVRS2VvdjBnQllOSmJOcHRkYl8yNlF1c0RCY3E2ckZkWHFBUmtERVgwSHUxT2pIS1VWb1FFZnREa2I?oc=5</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>taxi-point.co.uk</t>
+          <t>ACCESS Newswire</t>
         </is>
       </c>
       <c r="O24" s="2" t="b">
@@ -2161,31 +2161,31 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 19:38:27</t>
+          <t>2026-08-16 17:51:45</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>FSLR</t>
+          <t>HUM</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>First Solar</t>
+          <t>Humana</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>FSLR Stockholders Have Opportunity to Lead First Solar, Inc. Class Action Lawsuit – Contact Bronstein, Gewirtz and Grossman, LLC Today!</t>
+          <t>Glenmark USA Agrees to USD 15.28 Mn Settlement With Humana Over Generic Drug Antitrust Claims</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>FSLR 股東有機會領導 First Solar, Inc. 集體訴訟 – 立即聯繫 Bronstein、Gewirtz 和 Grossman, LLC！</t>
+          <t>Glenmark USA 同意就彷製藥反壟斷索賠與 Humana 達成 1528 萬美元和解</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.053</v>
+        <v>0.893</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
@@ -2194,12 +2194,12 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>MAJOR_LITIGATION</t>
+          <t>REGULATORY_PENALTY</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>重大訴訟</t>
+          <t>監管裁罰</t>
         </is>
       </c>
       <c r="J25" s="2" t="n">
@@ -2212,17 +2212,17 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>class action</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPYTRpVkpjZkxxY0JlcS1TeUVvaGRDRzUtMzFDMFFGRUZkYjNQMWFLOUVjdjFlNUdsMUNsRE5ZSWhUTHJYcEdNQmxuUFM4TC1PNENMTUQ1WVJDTk9YcmlGY0szRThtdHM3ZXFUVy1BcGhfQnB1RW1zNWtDTHk4ek94MzZ3bzBFbkdZZHFZZzNjMXI4b2FsQXpEUkktMF9iTUVwSWVSMEducmExRGVRS2VvdjBnQllOSmJOcHRkYl8yNlF1c0RCY3E2ckZkWHFBUmtERVgwSHUxT2pIS1VWb1FFZnREa2I?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOUjItZ3hfdEZDODdPQzd1MEVrMTdUOGpTbGRZTkhvS0IxbDZHZXJwbm1PR1pCYkFrWFRPdVAwR08yWktVa1pNcWhsTzE3TUo4RTZOeDhURUpiblZob05qQmlrY0xRT2c5aHBxVVkwMlVpcWVReUZKVkNVSjJkODIzOUVNblVSVU5XR3VJeE5mODhQbzI1NTVlcXZaYXJDcnRvTzFvWVVWNFRHeDctUGtzZlBfS2JqYmdnSjNlMWpTZDVwOXBqLVlfVEFWb3ZWa3cxc2NjX2F0NzdKbUUtQ01xM0530gHnAUFVX3lxTE5UWGJ0ODBjNThSeUhmLXM3SGtqU0ppSVM4LXhlNWtRd1YwNGpxcmd4Z3dyd25xVmx6QmFIb1MxM1RLaGxDOUk4SmkzSkVfaHZ4LU9nQkRnSUx5dGZwOE1JMlpybGZSQWptRi1vRWJ6Q2owUUFQc28zVjJNa2NXU2tmZXROSjkwcW93U3I1aVFHT1I1VU5ZS0NIRFVyd0d4NDhYMEtndlhmQ1lMSG9BaVNqNTdhNXctNHdtVmFLOWtKWlNtMDVmbDlyOHFDbDhoeFdBcTdWR1E3Ukx5QnFNMmFVYlRHZUFjRQ?oc=5</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>ACCESS Newswire</t>
+          <t>Medical Dialogues</t>
         </is>
       </c>
       <c r="O25" s="2" t="b">
@@ -2232,31 +2232,31 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 17:51:45</t>
+          <t>2026-08-16 15:26:00</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>HUM</t>
+          <t>IP</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Humana</t>
+          <t>International Paper</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Glenmark USA Agrees to USD 15.28 Mn Settlement With Humana Over Generic Drug Antitrust Claims</t>
+          <t>Phinge &amp; CEO Robert DeMaio Publicly Declare Cash Settlements or Judgments Alone Cannot &amp; Will Not Remedy the Deep Public Harm of Infringing Its IP</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Glenmark USA 同意就彷製藥反壟斷索賠與 Humana 達成 1528 萬美元和解</t>
+          <t>Phinge 及其執行長 Robert DeMaio 公開宣布僅靠現金和解或判決不能也不會彌補侵犯其智慧財產權所造成的深刻公共傷害</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.893</v>
+        <v>-0.889</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
@@ -2288,12 +2288,12 @@
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOUjItZ3hfdEZDODdPQzd1MEVrMTdUOGpTbGRZTkhvS0IxbDZHZXJwbm1PR1pCYkFrWFRPdVAwR08yWktVa1pNcWhsTzE3TUo4RTZOeDhURUpiblZob05qQmlrY0xRT2c5aHBxVVkwMlVpcWVReUZKVkNVSjJkODIzOUVNblVSVU5XR3VJeE5mODhQbzI1NTVlcXZaYXJDcnRvTzFvWVVWNFRHeDctUGtzZlBfS2JqYmdnSjNlMWpTZDVwOXBqLVlfVEFWb3ZWa3cxc2NjX2F0NzdKbUUtQ01xM0530gHnAUFVX3lxTE5UWGJ0ODBjNThSeUhmLXM3SGtqU0ppSVM4LXhlNWtRd1YwNGpxcmd4Z3dyd25xVmx6QmFIb1MxM1RLaGxDOUk4SmkzSkVfaHZ4LU9nQkRnSUx5dGZwOE1JMlpybGZSQWptRi1vRWJ6Q2owUUFQc28zVjJNa2NXU2tmZXROSjkwcW93U3I1aVFHT1I1VU5ZS0NIRFVyd0d4NDhYMEtndlhmQ1lMSG9BaVNqNTdhNXctNHdtVmFLOWtKWlNtMDVmbDlyOHFDbDhoeFdBcTdWR1E3Ukx5QnFNMmFVYlRHZUFjRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAJBVV95cUxNaTYyTlpabThoQlVfdTVhSEQ1TUM0bDNLNFk0NElFQnhOd1FueXZnRkp2U1RhcTIxTEl4WHFGUERkQTg5bGxVTDU4LWNGRnVHWGFPYmdING9NTEtrZmdLYVhqWFcza3hHc1NJTEQ3LXVEVngtc0tMUHU1QjZOYnhHbXhxU1BnMEV5TG9XdFMwQ1pHNHJXUHBEM3V4a3hSZ1N5ZnFlbnExWG12U1c4MExEa2VBbGdZeDVmSDhlY25EVEFWZ25EZGFDWm1ZS2l3aGtuMTlXSGJxV2doRzM2NFdnQWFrd2FoTEVySlVUZ0VRdHktS2R3S2hhMVJuWFFFMzgzanotSXNmMGdNVnZWZ09zeE43aVZ5RjFTUFI3LVNFa09RR1V6NWd3Tkg1QlAwSlhZ?oc=5</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>Medical Dialogues</t>
+          <t>FinancialContent</t>
         </is>
       </c>
       <c r="O26" s="2" t="b">
@@ -2303,31 +2303,31 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 15:26:00</t>
+          <t>2026-08-16 10:54:00</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>IP</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>International Paper</t>
+          <t>CF Industries</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Phinge &amp; CEO Robert DeMaio Publicly Declare Cash Settlements or Judgments Alone Cannot &amp; Will Not Remedy the Deep Public Harm of Infringing Its IP</t>
+          <t>Nashville SC - Inter Miami CF 1 - 0 | MISSED PENALTY - Leo Messi</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Phinge 及其執行長 Robert DeMaio 公開宣布僅靠現金和解或判決不能也不會彌補侵犯其智慧財產權所造成的深刻公共傷害</t>
+          <t>納許維爾 SC - 國際邁阿密 CF 1 - 0 |射失點球——裡奧梅西</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>-0.889</v>
+        <v>-0.237</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -2354,17 +2354,17 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>penalty</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAJBVV95cUxNaTYyTlpabThoQlVfdTVhSEQ1TUM0bDNLNFk0NElFQnhOd1FueXZnRkp2U1RhcTIxTEl4WHFGUERkQTg5bGxVTDU4LWNGRnVHWGFPYmdING9NTEtrZmdLYVhqWFcza3hHc1NJTEQ3LXVEVngtc0tMUHU1QjZOYnhHbXhxU1BnMEV5TG9XdFMwQ1pHNHJXUHBEM3V4a3hSZ1N5ZnFlbnExWG12U1c4MExEa2VBbGdZeDVmSDhlY25EVEFWZ25EZGFDWm1ZS2l3aGtuMTlXSGJxV2doRzM2NFdnQWFrd2FoTEVySlVUZ0VRdHktS2R3S2hhMVJuWFFFMzgzanotSXNmMGdNVnZWZ09zeE43aVZ5RjFTUFI3LVNFa09RR1V6NWd3Tkg1QlAwSlhZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE93ZXBzR2FQWGRhNnp4dlZKVnhyc0h2ZEJZNGRuRHFFUHRIVGlzQUZCNl9PYW1KMVFCeEV1cG14ZEM1UURyMmdIbHdHNktjZXJmeW9XWnpWUVNfeDdBUWxNYzhsTGk1T0JoQ0drYWlVcGc3MG00bkhFRDA4ckZEZ0E?oc=5</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>FinancialContent</t>
+          <t>Yahoo Sports</t>
         </is>
       </c>
       <c r="O27" s="2" t="b">
@@ -2374,68 +2374,68 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 10:54:00</t>
+          <t>2026-08-17 08:43:59</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>CF Industries</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Nashville SC - Inter Miami CF 1 - 0 | MISSED PENALTY - Leo Messi</t>
+          <t>IBM: ASEAN data breach costs hit record US$4.12 million as AI attacks rise</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>納許維爾 SC - 國際邁阿密 CF 1 - 0 |射失點球——裡奧梅西</t>
+          <t>IBM：隨著人工智慧攻擊的增加，東協資料外洩成本達到創紀錄的 412 萬美元</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>-0.237</v>
+        <v>0.306</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>LEGAL</t>
+          <t>CYBER</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>REGULATORY_PENALTY</t>
+          <t>DATA_BREACH</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>監管裁罰</t>
+          <t>資料外洩</t>
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>通知、檢視授信及自營部位、持續追蹤</t>
+          <t>通知、檢視授信及自營部位、加入觀察</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>penalty</t>
+          <t>data breach</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE93ZXBzR2FQWGRhNnp4dlZKVnhyc0h2ZEJZNGRuRHFFUHRIVGlzQUZCNl9PYW1KMVFCeEV1cG14ZEM1UURyMmdIbHdHNktjZXJmeW9XWnpWUVNfeDdBUWxNYzhsTGk1T0JoQ0drYWlVcGc3MG00bkhFRDA4ckZEZ0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPNUVuMF9LcEVmNW10UFR0elo3Y2syYzdOaWZuMkh0N01EaW9oNVg1NmpTWk9xMjRESnVNcnBvTXZ5eXZBWFVEOEFXZHlkNjdybF9xSFlERUtrd0hJalhLSkxwbFZjZDlSQUxnOFZDVEdCeHBSLW1aZmlsNjNMX0ZRQzdKRWZldDZpenlsV0FqVFlxUkhkMnc?oc=5</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports</t>
+          <t>crnasia.com</t>
         </is>
       </c>
       <c r="O28" s="2" t="b">
@@ -2445,45 +2445,45 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:43:59</t>
+          <t>2026-08-17 08:38:35</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>IBM: ASEAN data breach costs hit record US$4.12 million as AI attacks rise</t>
+          <t>Boeing Classic: Stewart Cink defeats Miguel Angel Jimenez in playoff</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>IBM：隨著人工智慧攻擊的增加，東協資料外洩成本達到創紀錄的 412 萬美元</t>
+          <t>波音經典賽：史都華辛克在延長賽中擊敗米格爾安赫爾希門尼斯</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.306</v>
+        <v>0.089</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>CYBER</t>
+          <t>OPERATIONS</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>DATA_BREACH</t>
+          <t>WORKFORCE_REDUCTION</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>資料外洩</t>
+          <t>裁員或人力縮減</t>
         </is>
       </c>
       <c r="J29" s="2" t="n">
@@ -2496,17 +2496,17 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>data breach</t>
+          <t>layoff</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPNUVuMF9LcEVmNW10UFR0elo3Y2syYzdOaWZuMkh0N01EaW9oNVg1NmpTWk9xMjRESnVNcnBvTXZ5eXZBWFVEOEFXZHlkNjdybF9xSFlERUtrd0hJalhLSkxwbFZjZDlSQUxnOFZDVEdCeHBSLW1aZmlsNjNMX0ZRQzdKRWZldDZpenlsV0FqVFlxUkhkMnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxQYWZuLTJVelJiN2hGeW5tYU4tc2g2c281Vm9QOFpVQzB0VDBPTDNOSjRBb0Zac1M2MjllcGdySXpoT0pNcXpKclZocnVFeFFGLUNvemtKdzd0VEFxZHlNMTUzRGsxUEtGanhISGNsS2NwUk9aaXJkWFo3QkwwajZ4Y3FrZlBlUzdUMVV1d1lpclBaWVlQVEJ2anVoOHNZLV9PWTlMeDltZzl3ZzhoVnc?oc=5</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>CRN Asia</t>
+          <t>The Seattle Times</t>
         </is>
       </c>
       <c r="O29" s="2" t="b">
@@ -2516,31 +2516,31 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:38:35</t>
+          <t>2026-08-17 08:25:01</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>FedEx</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Boeing Classic: Stewart Cink defeats Miguel Angel Jimenez in playoff</t>
+          <t>Scheffler wins FedEx Cup playoff opener in a runaway and Jack Whaley claims the U.S. Amateur</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>波音經典賽：史都華辛克在延長賽中擊敗米格爾安赫爾希門尼斯</t>
+          <t>舍夫勒在聯邦快遞杯季後賽首戰大獲全勝，傑克威利奪得美國業餘冠軍</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.089</v>
+        <v>0.302</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -2572,12 +2572,12 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxQYWZuLTJVelJiN2hGeW5tYU4tc2g2c281Vm9QOFpVQzB0VDBPTDNOSjRBb0Zac1M2MjllcGdySXpoT0pNcXpKclZocnVFeFFGLUNvemtKdzd0VEFxZHlNMTUzRGsxUEtGanhISGNsS2NwUk9aaXJkWFo3QkwwajZ4Y3FrZlBlUzdUMVV1d1lpclBaWVlQVEJ2anVoOHNZLV9PWTlMeDltZzl3ZzhoVnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxQMnlBeGFWNUMxdzBaSzN3NlJDZWc5OVBtb25fZk8yWFZ2Mi1EanhjLW9neVFtaFhwVEZKY21SS1pUakdRQkx4cEhmZlc4V0s3WjFxZnQ2ZnUwYXpvRWxJWDdfdlEzbHZoM0xtUVFfMUoybXU4WTlQUTlncnFiWG15TGpQWFQyM3hva29sTWp0b0JQbGR0MHdiWXJnU1RTLXVObFNkcXNoWWtUWWt4eEdGUU81OFV1aldzeFdLd2dSc0p0Z1VjYjk0cUFJdFNnV3VhVXNWTHZmMzV3Zkt5UV9iMFNNcXl3NWV4QmpQOVdzSUlCUDVmX1hmaEpvSF9oWU9pSXNMdzNfWQ?oc=5</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>The Seattle Times</t>
+          <t>messenger-inquirer.com</t>
         </is>
       </c>
       <c r="O30" s="2" t="b">
@@ -2587,7 +2587,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:25:00</t>
+          <t>2026-08-17 08:24:45</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2602,16 +2602,16 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Scheffler wins FedEx Cup playoff opener in a runaway and Jack Whaley claims the U.S. Amateur</t>
+          <t>Jordan Spieth's season ends after being narrowly eliminated from FedEx Cup playoffs</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>舍夫勒在聯邦快遞杯季後賽首戰大獲全勝，傑克威利奪得美國業餘冠軍</t>
+          <t>喬丹史匹斯在聯邦快遞杯季後賽以微弱優勢被淘汰後賽季結束</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.302</v>
+        <v>-0.903</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -2638,12 +2638,12 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>layoff</t>
+          <t>layoff；layoffs</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQUV9od29DanJDbmdGeDJjUXIyV0o0eHZ6U1FLZEhxNEoyNThsMnI2YTk4UFBCczFqWjg0dm9GazI0aU10aDMyeTFHT1VLZUpLZ3FoZTNhcmhvLXFWeWJPeU9rUnlGeTktZ1JlMmNHemRHMnVKY1IxaWhQVjBNYUpUbmhHSU9ERWF3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQcGl3RFlpanRXV3NtSHdROUNXZENHXzdOalotcWZFWGwtQ0JVS3pBa05CRzVFRnpqb29JT1c3Qkhpc2FfY2ltYS1Sb0c1bmUyYmZ3YlBkRnVMVVRQazdOM3NIS0haWkxXT2xZX3c3NzE5eVNjNGFmVFh4X2ZCaXJsWEY3bVNPYXhC?oc=5</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
@@ -2658,31 +2658,31 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:24:45</t>
+          <t>2026-08-17 08:21:43</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>KIM</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>FedEx</t>
+          <t>Kimco Realty</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Jordan Spieth's season ends after being narrowly eliminated from FedEx Cup playoffs</t>
+          <t>Kim Si-woo Runner-Up as All Three Koreans Advance in PGA Playoffs</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>喬丹史匹斯在聯邦快遞杯季後賽以微弱優勢被淘汰後賽季結束</t>
+          <t>金時宇獲得亞軍，三位韓國選手全數晉級 PGA 季後賽</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>-0.903</v>
+        <v>0.773</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
@@ -2714,12 +2714,12 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQcGl3RFlpanRXV3NtSHdROUNXZENHXzdOalotcWZFWGwtQ0JVS3pBa05CRzVFRnpqb29JT1c3Qkhpc2FfY2ltYS1Sb0c1bmUyYmZ3YlBkRnVMVVRQazdOM3NIS0haWkxXT2xZX3c3NzE5eVNjNGFmVFh4X2ZCaXJsWEY3bVNPYXhC?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOeUR2Y3ZGM2FidU1tNmtrcEJDQkhJZzVwY0VFeWREQld2SDlWZlNNTzc4T2luRm9RV3RCMXRIUHJQYUhMY0pUVDNnd0V6S1k4VEFfcGUyZF9iY09MSkdaTnlZbGszUDk3R1FXd0Iza0d2R1VTOVVVTTY2aUdQdE00cmZVMUlGVm1aYTdDbXJVT21vRGxCX2oxRW5xeGNaUQ?oc=5</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports</t>
+          <t>en.sedaily.com</t>
         </is>
       </c>
       <c r="O32" s="2" t="b">
@@ -2729,31 +2729,31 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:21:43</t>
+          <t>2026-08-17 07:54:18</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>KIM</t>
+          <t>CCL</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Kimco Realty</t>
+          <t>Carnival Corporation</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Kim Si-woo Runner-Up as All Three Koreans Advance in PGA Playoffs</t>
+          <t>AI server tracker: Demand drives strong growth across Taiwan's CCL, design services, substrate, and testing supply chains</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>金時宇獲得亞軍，三位韓國選手全數晉級 PGA 季後賽</t>
+          <t>AI伺服器追蹤器：需求推動台灣覆銅板、設計服務、基板和測試供應鏈的強勁成長</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.773</v>
+        <v>0.929</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -2762,12 +2762,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>WORKFORCE_REDUCTION</t>
+          <t>SUPPLY_CHAIN_DISRUPTION</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>裁員或人力縮減</t>
+          <t>供應鏈中斷</t>
         </is>
       </c>
       <c r="J33" s="2" t="n">
@@ -2780,17 +2780,17 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>layoff；layoffs</t>
+          <t>supply chain</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOeUR2Y3ZGM2FidU1tNmtrcEJDQkhJZzVwY0VFeWREQld2SDlWZlNNTzc4T2luRm9RV3RCMXRIUHJQYUhMY0pUVDNnd0V6S1k4VEFfcGUyZF9iY09MSkdaTnlZbGszUDk3R1FXd0Iza0d2R1VTOVVVTTY2aUdQdE00cmZVMUlGVm1aYTdDbXJVT21vRGxCX2oxRW5xeGNaUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPYVl0V1kyY0RlUjFnSnFtdFo0MDd3ZUR5c0JtVV9pUUpDVVpZTHR1QmlPY1Jtb1RCWVpIVGFpQVBZUWJ4UE5Fejk5YXpSREhxdXQwdzVWMXp1b3F0d0xpYTBUN210cE1XWEJLOHVHaVZndHowN3o3dUViN2V3OEcwdGdRbDdwMmhPaHdHVXdVSXk3T1pDTFZHSFBWSGpmYVZtSWVUbg?oc=5</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Seoul Economic Daily</t>
+          <t>digitimes</t>
         </is>
       </c>
       <c r="O33" s="2" t="b">
@@ -2800,31 +2800,31 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 07:54:18</t>
+          <t>2026-08-17 07:33:00</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>CCL</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Carnival Corporation</t>
+          <t>FedEx</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>AI server tracker: Demand drives strong growth across Taiwan's CCL, design services, substrate, and testing supply chains</t>
+          <t>Who was eliminated from golf's FedExCup Playoffs? Jordan Spieth leads list</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>AI伺服器追蹤器：需求推動台灣覆銅板、設計服務、基板和測試供應鏈的強勁成長</t>
+          <t>誰在高爾夫聯邦快遞杯季後賽中被淘汰？喬丹·斯皮思領先榜單</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.929</v>
+        <v>-0.434</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
@@ -2833,12 +2833,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>SUPPLY_CHAIN_DISRUPTION</t>
+          <t>WORKFORCE_REDUCTION</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>供應鏈中斷</t>
+          <t>裁員或人力縮減</t>
         </is>
       </c>
       <c r="J34" s="2" t="n">
@@ -2851,17 +2851,17 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>supply chain</t>
+          <t>layoff；layoffs</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPYVl0V1kyY0RlUjFnSnFtdFo0MDd3ZUR5c0JtVV9pUUpDVVpZTHR1QmlPY1Jtb1RCWVpIVGFpQVBZUWJ4UE5Fejk5YXpSREhxdXQwdzVWMXp1b3F0d0xpYTBUN210cE1XWEJLOHVHaVZndHowN3o3dUViN2V3OEcwdGdRbDdwMmhPaHdHVXdVSXk3T1pDTFZHSFBWSGpmYVZtSWVUbg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOV1ZCWjRfYXh3T1JVTFN0Q2pYS2VEVHN2TC1GaVNodG54RndmcU1XZHdsZUVDajRuR2J6VWo5SDlKSUN1c3d0eXJPS1lnV0RmS1I3Y08tZ1cyTkhCbEFuWXFHaVVKLTFKVXlkcXQ0bEJERENpVV9SMEptSlpXWnpVaWhFTEVZNkFRYm53RlgwMTdCc1lTY0VVejhNOFlwc19aMmVsRDczNVJVcXR6QnR3dElMSVV3cUpKOV8xMw?oc=5</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>digitimes</t>
+          <t>USA Today</t>
         </is>
       </c>
       <c r="O34" s="2" t="b">
@@ -2871,7 +2871,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 07:33:00</t>
+          <t>2026-08-17 07:10:00</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2886,16 +2886,16 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Who was eliminated from golf's FedExCup Playoffs? Jordan Spieth leads list</t>
+          <t>Jordan Spieth, Keith Mitchell among the 20 exiting FedEx Playoffs before BMW</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>誰在高爾夫聯邦快遞杯季後賽中被淘汰？喬丹·斯皮思領先榜單</t>
+          <t>喬丹史匹斯 (Jordan Spieth)、基斯米切爾 (Keith Mitchell) 躋身聯邦快遞季後賽前 20 名，排在寶馬之前</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>-0.434</v>
+        <v>-0.011</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
@@ -2927,12 +2927,12 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOV1ZCWjRfYXh3T1JVTFN0Q2pYS2VEVHN2TC1GaVNodG54RndmcU1XZHdsZUVDajRuR2J6VWo5SDlKSUN1c3d0eXJPS1lnV0RmS1I3Y08tZ1cyTkhCbEFuWXFHaVVKLTFKVXlkcXQ0bEJERENpVV9SMEptSlpXWnpVaWhFTEVZNkFRYm53RlgwMTdCc1lTY0VVejhNOFlwc19aMmVsRDczNVJVcXR6QnR3dElMSVV3cUpKOV8xMw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxNTXhjdWlJOFc5VFRIMlpja2FtaWNxeW5JLVF6WW5jRWU3em5qcnVZaEljTlR2S2piLWpCSEtCYVBENTkyUE1Nc0hHektBWWloMGpCdmt3NXpfSUhza244cHNaRzZVcWdxX0o3cUl4OHNMVmlvdkwwbXEyb2ppNzhZY1B3eGpibmNlYXNrMkNWVlhuT0hzazlQMUF6TzBsN25VVlhiU05FZjFEeEF1QjI4dHc3UzRVVkJxTU5jbmowMTNFV0tIZWlJRnhUV3FnTVZDVURSRXhGNXloUkhqOUpkY29yTkw?oc=5</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>USA Today</t>
+          <t>Golfweek</t>
         </is>
       </c>
       <c r="O35" s="2" t="b">
@@ -2942,7 +2942,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 07:10:00</t>
+          <t>2026-08-17 07:08:00</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2957,16 +2957,16 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Jordan Spieth, Keith Mitchell among the 20 exiting FedEx Playoffs before BMW</t>
+          <t>See the top 50 in FedEx Cup Playoffs standings heading to the BMW Championship</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>喬丹史匹斯 (Jordan Spieth)、基斯米切爾 (Keith Mitchell) 躋身聯邦快遞季後賽前 20 名，排在寶馬之前</t>
+          <t>查看聯邦快遞杯季後賽積分榜前 50 名，前往 BMW 錦標賽</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>-0.011</v>
+        <v>0.178</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxNTXhjdWlJOFc5VFRIMlpja2FtaWNxeW5JLVF6WW5jRWU3em5qcnVZaEljTlR2S2piLWpCSEtCYVBENTkyUE1Nc0hHektBWWloMGpCdmt3NXpfSUhza244cHNaRzZVcWdxX0o3cUl4OHNMVmlvdkwwbXEyb2ppNzhZY1B3eGpibmNlYXNrMkNWVlhuT0hzazlQMUF6TzBsN25VVlhiU05FZjFEeEF1QjI4dHc3UzRVVkJxTU5jbmowMTNFV0tIZWlJRnhUV3FnTVZDVURSRXhGNXloUkhqOUpkY29yTkw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPdFN1RUpYWnpYdndUSldsNWVJTmVIaDVpNkRfbGlQRzhZVkl5aXVGaWw0MVhBcFFjUmsyR1gxVkNIcXhITzc4Q2hxYk1OMUtYYk5HLU8wQXpvU01hNTRweng2dm5rT2Q3MXZ2bTlhbXRiYW1Ha3VRLUJERXRha0lrY1dVRlFxZDQ5XzdPRU5SRDUwN0RZWUxOcUt5bU9yakR0QW9PczZLS2o0bTFEVXpnNDFnLU5UNHBuejQyWlNoNjZXWkpRMEoxYTNIcldTUWNBVVVvRHNNQXJla3ZIWkVzRF92aFkwOFFteEpPcA?oc=5</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
@@ -3013,31 +3013,31 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 07:08:00</t>
+          <t>2026-08-17 06:49:24</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>FedEx</t>
+          <t>Goldman Sachs</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>See the top 50 in FedEx Cup Playoffs standings heading to the BMW Championship</t>
+          <t>Goldman Sachs Alternatives To Acquire Tosca From Apax, Backing 63-Center Reusable Food Supply Chain Platform</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>查看聯邦快遞杯季後賽積分榜前 50 名，前往 BMW 錦標賽</t>
+          <t>高盛Alternatives將從Apax手中收購Tosca，支援63中心可重複使用食品供應鏈平台</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.178</v>
+        <v>0.437</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -3046,12 +3046,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>WORKFORCE_REDUCTION</t>
+          <t>SUPPLY_CHAIN_DISRUPTION</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>裁員或人力縮減</t>
+          <t>供應鏈中斷</t>
         </is>
       </c>
       <c r="J37" s="2" t="n">
@@ -3064,17 +3064,17 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>layoff；layoffs</t>
+          <t>supply chain</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPdFN1RUpYWnpYdndUSldsNWVJTmVIaDVpNkRfbGlQRzhZVkl5aXVGaWw0MVhBcFFjUmsyR1gxVkNIcXhITzc4Q2hxYk1OMUtYYk5HLU8wQXpvU01hNTRweng2dm5rT2Q3MXZ2bTlhbXRiYW1Ha3VRLUJERXRha0lrY1dVRlFxZDQ5XzdPRU5SRDUwN0RZWUxOcUt5bU9yakR0QW9PczZLS2o0bTFEVXpnNDFnLU5UNHBuejQyWlNoNjZXWkpRMEoxYTNIcldTUWNBVVVvRHNNQXJla3ZIWkVzRF92aFkwOFFteEpPcA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxPeWQ0UzE3NzBYTzhBRVNKQTludUl3Q2N4ckdqTEZmR3hUcmJqSHFiR0V2YWNLSXRWMmNIVnVNYTFZYWUxLW5iYVhKT1Zvb3pvSkJRd3FaYS1PT1EtUWVLbUxRRGx6dkktVE5ObjlXQ1BuczFqVWFBcHVWYzlOOWxQckYySVUxQ1liR25GSklXTHZNZ25taExUSExDcVV6Q2lyelJPeHZQd1VxQ0tUaGFsZnVodVRkdzRSR2E5X1g2WWxxeEFMWkHSAcsBQVVfeXFMTk9jbUZrUk1PeVpfRm8wMlNuRm85czVNc2JyZXlzeTNzcS02YnZtd1J0X0Fod29OazNRTEhQeUtLWFJkbTlzWTBGSWg1NjVJdEpKN0dpRzl5cXZncWhBWjVnd3BtX20tMk1xYzlUWmIxNjIyTElRaVZFWE1DSnJMamxyanNaeGpHbVlicnJLYXBSZ0NSeGF4YkFPaTVNdHdUcmZyRjZ5Um1ONXlPQmhQMERrc2dqZlFvZmV5VjNPV0Y2WnNzYmttV0pWLW8?oc=5</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>Golfweek</t>
+          <t>Pulse 2.0</t>
         </is>
       </c>
       <c r="O37" s="2" t="b">
@@ -3084,31 +3084,31 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 06:49:24</t>
+          <t>2026-08-17 06:49:00</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>KIM</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Goldman Sachs</t>
+          <t>Kimco Realty</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Goldman Sachs Alternatives To Acquire Tosca From Apax, Backing 63-Center Reusable Food Supply Chain Platform</t>
+          <t>Kim Si-woo Finishes Runner-Up at PGA Tour Playoff Opener, Advances to Round 2 with Im Sung-jae and Kim Joo-hyung</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>高盛Alternatives將從Apax手中收購Tosca，支援63中心可重複使用食品供應鏈平台</t>
+          <t>金時宇在PGA巡迴賽季後賽揭幕戰中獲得亞軍，與林成宰和金珠亨一起晉級第二輪</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.437</v>
+        <v>0.423</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -3117,12 +3117,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>SUPPLY_CHAIN_DISRUPTION</t>
+          <t>WORKFORCE_REDUCTION</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>供應鏈中斷</t>
+          <t>裁員或人力縮減</t>
         </is>
       </c>
       <c r="J38" s="2" t="n">
@@ -3135,17 +3135,17 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>supply chain</t>
+          <t>layoff</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxPeWQ0UzE3NzBYTzhBRVNKQTludUl3Q2N4ckdqTEZmR3hUcmJqSHFiR0V2YWNLSXRWMmNIVnVNYTFZYWUxLW5iYVhKT1Zvb3pvSkJRd3FaYS1PT1EtUWVLbUxRRGx6dkktVE5ObjlXQ1BuczFqVWFBcHVWYzlOOWxQckYySVUxQ1liR25GSklXTHZNZ25taExUSExDcVV6Q2lyelJPeHZQd1VxQ0tUaGFsZnVodVRkdzRSR2E5X1g2WWxxeEFMWkHSAcsBQVVfeXFMTk9jbUZrUk1PeVpfRm8wMlNuRm85czVNc2JyZXlzeTNzcS02YnZtd1J0X0Fod29OazNRTEhQeUtLWFJkbTlzWTBGSWg1NjVJdEpKN0dpRzl5cXZncWhBWjVnd3BtX20tMk1xYzlUWmIxNjIyTElRaVZFWE1DSnJMamxyanNaeGpHbVlicnJLYXBSZ0NSeGF4YkFPaTVNdHdUcmZyRjZ5Um1ONXlPQmhQMERrc2dqZlFvZmV5VjNPV0Y2WnNzYmttV0pWLW8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE1OMnVlcjhiNmZXUFRzcHRrWFhuMDlrTDg0a1BDSmxvNXhnalkzUl93eHlGa0Q5ZU92b2c5V1gyWXhZYzh4R1Aya1kyam5KZzNWZXJVZ3ZJbUE4MEU1UTdpRHhiVWZxUQ?oc=5</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>Pulse 2.0</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="O38" s="2" t="b">
@@ -3155,31 +3155,31 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 06:49:00</t>
+          <t>2026-08-17 06:41:28</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>KIM</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Kimco Realty</t>
+          <t>FedEx</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Kim Si-woo Finishes Runner-Up at PGA Tour Playoff Opener, Advances to Round 2 with Im Sung-jae and Kim Joo-hyung</t>
+          <t>FedEx Cup 2026 Points, Playoff Standings After St. Jude Championship</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>金時宇在PGA巡迴賽季後賽揭幕戰中獲得亞軍，與林成宰和金珠亨一起晉級第二輪</t>
+          <t>聖裘德錦標賽後 2026 年聯邦快遞杯積分、季後賽積分榜</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.423</v>
+        <v>0.101</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -3211,12 +3211,12 @@
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE1OMnVlcjhiNmZXUFRzcHRrWFhuMDlrTDg0a1BDSmxvNXhnalkzUl93eHlGa0Q5ZU92b2c5V1gyWXhZYzh4R1Aya1kyam5KZzNWZXJVZ3ZJbUE4MEU1UTdpRHhiVWZxUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNcHVxenIwSGJJMGp4eW4wTFhjbV9sdGZmZzlyNlFzdGtIUURMbUF5LTU5SUlYQmtaN29QZGFKV1h3c3kyUDBQUW5xdTdXMVVGNjgtQmxSbEFvM3FzSHh4dVRGelktNGdKbWtHZ2RWOHkxSDJBeU1FSnRZRHZfT3NvVjhFZ1htOGJSR050WWRuUGQ0QTB5YVNyX1dPblIyZnFkcXVNTUdqZ3hhWFRBUTl1WA?oc=5</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>Bleacher Report</t>
         </is>
       </c>
       <c r="O39" s="2" t="b">
@@ -3226,7 +3226,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 06:41:28</t>
+          <t>2026-08-17 06:33:54</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3241,16 +3241,16 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>FedEx Cup 2026 Points, Playoff Standings After St. Jude Championship</t>
+          <t>Collin Morikawa is Lone Ex-Cal Golfer Still Alive in FedEx Cup Playoffs</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>聖裘德錦標賽後 2026 年聯邦快遞杯積分、季後賽積分榜</t>
+          <t>科林森川是聯邦快遞杯季後賽中唯一仍然活著的前加州高爾夫球手</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.101</v>
+        <v>0.018</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
@@ -3277,17 +3277,17 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>layoff</t>
+          <t>layoff；layoffs</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNcHVxenIwSGJJMGp4eW4wTFhjbV9sdGZmZzlyNlFzdGtIUURMbUF5LTU5SUlYQmtaN29QZGFKV1h3c3kyUDBQUW5xdTdXMVVGNjgtQmxSbEFvM3FzSHh4dVRGelktNGdKbWtHZ2RWOHkxSDJBeU1FSnRZRHZfT3NvVjhFZ1htOGJSR050WWRuUGQ0QTB5YVNyX1dPblIyZnFkcXVNTUdqZ3hhWFRBUTl1WA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQbGplTFY4cU5ncHJmaEozUktLMFhKR3FueUFhSktIaW9QVE1CUFRIY1lfZVVrUm1jRXdZYjJZSHNXQV9oMzJVRU10dWpWbFg3NGxKLWFUSFBUSjV1VGZVTG9UTktpdU5vdjh0OHBjU28xV3JvclB5emxOUHVCb0RTYTNubTJGV2s5NWZWekU5MGR1TjNGcUNKbjJRakxFMUljOG5NcFBBamVMTk1Db2h3S0tSN0RQOTJLTEhyTjlZN2g2dmlGdVJN?oc=5</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>bleacherreport.com</t>
+          <t>si.com</t>
         </is>
       </c>
       <c r="O40" s="2" t="b">
@@ -3297,31 +3297,31 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 06:33:54</t>
+          <t>2026-08-17 06:24:50</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>FedEx</t>
+          <t>Hasbro</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Collin Morikawa is Lone Ex-Cal Golfer Still Alive in FedEx Cup Playoffs</t>
+          <t>Rory McIlroy has rough week, posts worst finish of the season at FedEx St. Jude Championship to open playoffs</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>科林森川是聯邦快遞杯季後賽中唯一仍然活著的前加州高爾夫球手</t>
+          <t>羅裡·麥克羅伊度過了艱難的一周，在聯邦快遞聖裘德錦標賽季後賽中取得了本賽季最差的成績</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0.018</v>
+        <v>-0.9350000000000001</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
@@ -3353,7 +3353,7 @@
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQaEJDeG9CM0NrTndKNDRLZTlqN1pqYVZVTDZ5M190bTZQbzQwc29zT3NSVXQ5OGdOYTNRSU8xNWx6MUJkQnJsVEJYazBUYUQwZy1XQ0h1WFBxaHBxb3o5WDVnbkk5bW8zMVc0ZUJwWnlnZURpOVpueDNUT2dfVDk4RGtR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQbEdPNVRrREFlMTB2TVRESzdibkZreTNJSlRtQlZ5YXNxU3QzbTRQeFRuNDlCMDJvNS1vdExzRXVwTGdKdTd2azAtaVd1aTRUNVF2NWM3SGVlcVdTS3lDc0tIRWNQOS1oWkFDcEJiN3ZremtQdjBxRDNKNkI4Zllic2hzYU00UE1SOC1pcFIwTU1aWjc2dDlYdXdQV054RmNtMXJOR0hSWWV3dFk5dVhfSHp5LTZxM0xjTFA2eDFpVUxJMzR5bV96cC1Tb1dZeFItWlBaLWFwaDNTemhncG5IcVpMbU9CSTlxSVlzQTliT3lxdw?oc=5</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
@@ -3439,31 +3439,31 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 06:24:50</t>
+          <t>2026-08-17 04:00:00</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Hasbro</t>
+          <t>FedEx</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Rory McIlroy has rough week, posts worst finish of the season at FedEx St. Jude Championship to open playoffs</t>
+          <t>2026 St. Jude Championship TV schedule, coverage: Where to watch first leg of FedEx Cup Playoffs</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>羅裡·麥克羅伊度過了艱難的一周，在聯邦快遞聖裘德錦標賽季後賽中取得了本賽季最差的成績</t>
+          <t>2026 年聖裘德錦標賽電視節目表、報導：在哪裡觀看聯邦快遞杯季後賽第一回合</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>-0.9350000000000001</v>
+        <v>-0.006</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -3495,12 +3495,12 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQbEdPNVRrREFlMTB2TVRESzdibkZreTNJSlRtQlZ5YXNxU3QzbTRQeFRuNDlCMDJvNS1vdExzRXVwTGdKdTd2azAtaVd1aTRUNVF2NWM3SGVlcVdTS3lDc0tIRWNQOS1oWkFDcEJiN3ZremtQdjBxRDNKNkI4Zllic2hzYU00UE1SOC1pcFIwTU1aWjc2dDlYdXdQV054RmNtMXJOR0hSWWV3dFk5dVhfSHp5LTZxM0xjTFA2eDFpVUxJMzR5bV96cC1Tb1dZeFItWlBaLWFwaDNTemhncG5IcVpMbU9CSTlxSVlzQTliT3lxdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQOHkxSGVRQzdhLUtGMl9CQWlLM05OVklfYk5hXzczZ0I2ajVfUl9RcDhkX19MLWhfWTVENHJmR19yXzZaNXVmZDQ5UGRUVldxNnVHTUpYM1BpUVNScXhzNmJxaENzNm96WkFqOXNpZkFYSjB2bFJ2eDdtM1lMSFBHWW96MU9zRDhmZm5XNEpGR1NWRHJJUk1DdF9nVzNBVVBIOW5fWU1lV2F6dzhUdTZxaE1XbWstZXBKZ3BFVkJoWkJGMUNQRkE?oc=5</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Sports</t>
+          <t>CBS Sports</t>
         </is>
       </c>
       <c r="O43" s="2" t="b">
@@ -3510,31 +3510,31 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 04:00:00</t>
+          <t>2026-08-17 03:38:53</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>FedEx</t>
+          <t>General Motors</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026 St. Jude Championship TV schedule, coverage: Where to watch first leg of FedEx Cup Playoffs</t>
+          <t>Aces Vs Liberty Gm 2 | 2024 WNBA Playoffs | WNBA Best Bets &amp; Predictions | ChrisBeCappinn Show Golshifteh Farahani (nfYEvsTvq9)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026 年聖裘德錦標賽電視節目表、報導：在哪裡觀看聯邦快遞杯季後賽第一回合</t>
+          <t>王牌 vs 自由 Gm 2 | 2024 年 WNBA 季後賽 | WNBA 最佳投注和預測 | ChrisBeCappinn 秀 Golshifteh Farahani (nfYEvsTvq9)</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>-0.006</v>
+        <v>0.014</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
@@ -3566,12 +3566,12 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQOHkxSGVRQzdhLUtGMl9CQWlLM05OVklfYk5hXzczZ0I2ajVfUl9RcDhkX19MLWhfWTVENHJmR19yXzZaNXVmZDQ5UGRUVldxNnVHTUpYM1BpUVNScXhzNmJxaENzNm96WkFqOXNpZkFYSjB2bFJ2eDdtM1lMSFBHWW96MU9zRDhmZm5XNEpGR1NWRHJJUk1DdF9nVzNBVVBIOW5fWU1lV2F6dzhUdTZxaE1XbWstZXBKZ3BFVkJoWkJGMUNQRkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTFBZLWVvZmg5YXhKZW5OM3hSZU1sNjBRd0RSRXJpRHRwTmZyV2RYelJucG9CMGlFQVhvUWNKdDBxOGNoWFJTWng0NFNZTHdicHYtY3JhVlpSZjBxZWxwR2xMSw?oc=5</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>CBS Sports</t>
+          <t>Mshale</t>
         </is>
       </c>
       <c r="O44" s="2" t="b">
@@ -3865,31 +3865,31 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 15:24:44</t>
+          <t>2026-08-16 16:03:58</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>COIN</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>Coinbase</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Stewart Cink beats Miguel Angel Jiménez in playoff to win Boeing Classic, earns fifth title of season</t>
+          <t>Bitcoin demand weakens as Coinbase premium inde...</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>史都華辛克在延長賽中擊敗米格爾安赫爾希門尼斯贏得波音精英賽冠軍，贏得本賽季第五個冠軍</t>
+          <t>隨著 Coinbase 溢價指數下降，比特幣需求減弱</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0.243</v>
+        <v>-0.947</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -3898,12 +3898,12 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>WORKFORCE_REDUCTION</t>
+          <t>OPERATING_DETERIORATION</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>裁員或人力縮減</t>
+          <t>營運惡化</t>
         </is>
       </c>
       <c r="J49" s="2" t="n">
@@ -3916,17 +3916,17 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>layoff</t>
+          <t>demand weakens</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOaUFhMGUxRXNPeDVmVjV2ajd5Y0VEMHQ3X3E1QVdkLWZYMnpOSjdqX281SjdCYmhkdXpRc1hSRXVoSkdweWs5OXVNa1NENHNpdWVWS25falJkM2FfcC1fUGR3alJKQ0R0QlU4eTFwZ0RVcVFFV1RqWkl5ZWNoV1dYZG1OeGRuZ05JUE11Q2ZjeHVhck8wRzFROFRHdGZIM0VKQ1Ytc2N0a0w0S0QzZlVEMWlnckVTRXFSQmNxZk8xU01NbDBnTE5OUUlIaU9KNFdBT3dPWW5Kb0lxdnZhX1RtR1REeWk2VG5qSDlyUDdrRFVtWHM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxQczhZLW84MjR0NmNrcVE5LVRvLW1LTm5xMDJxaUl6cXBfbERFV3R1N1ROa0p4RWExbkZuOVJQT19nWV93RWdJamtqNVY2bURoeUFUczdBY2J3eUJEVkhBTkE3dXNaUG9WYzdtVmdJSUhtSDlyRXR6b2JETU9zTVAzdDkyMmNFNTNTSGc?oc=5</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>PGA Tour</t>
+          <t>Pluang</t>
         </is>
       </c>
       <c r="O49" s="2" t="b">
@@ -3936,68 +3936,68 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 03:20:18</t>
+          <t>2026-08-16 15:24:44</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Deere &amp; Company</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Abelardo de la Espriella asks Donald Trump to suspend tariffs to help Colombia earthquake recovery</t>
+          <t>Stewart Cink beats Miguel Angel Jiménez in playoff to win Boeing Classic, earns fifth title of season</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>阿韋拉多·德拉埃斯普里埃拉要求唐納德·特朗普暫停關稅以幫助哥倫比亞地震恢復</t>
+          <t>史都華辛克在延長賽中擊敗米格爾安赫爾希門尼斯贏得波音精英賽冠軍，贏得本賽季第五個冠軍</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>-0.8080000000000001</v>
+        <v>0.243</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>GEOPOLITICAL</t>
+          <t>OPERATIONS</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>TARIFF</t>
+          <t>WORKFORCE_REDUCTION</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>關稅</t>
+          <t>裁員或人力縮減</t>
         </is>
       </c>
       <c r="J50" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>僅紀錄</t>
+          <t>通知、檢視授信及自營部位、加入觀察</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>tariff</t>
+          <t>layoff</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNVXhoZm85Q3Y5NklZRk8tUUJ6OGc3M2FNOWE0Z1pYWENfdmZVT0FUQ0h4SEJYcWc5THJjRjh3bW1xczhERElnNXpUVko0eEVZLVRLcWkwaTFDX3NBNGl2T1BnYldKVlFoZzltSlMyalVmMEJ2YmRrM19NN0lNQmZBNVp5THl1NERLT1BsMnA5ZXNkTXJUQlpReS1aNE5FXzQ0TVFqUTlsUzNaX0xMM0JsQzVlTkdvNE5OWW9Lb3NNcWJUNG9XSkJvM0xWd9IB0AFBVV95cUxQMU5vNHRDdjVYMEhQQnVvNVRPVTdZVmdBRm1zalNuYmlaSURqckF1NU5PVl9zV0ZSYngweG5KdjFaY25LekVYajFEWDZlQk01V2xTc0FkcGlnSGZWaXpjcV9hNkpzcndHSEZTNGtHTzJzZy0tN0pFYi1XM2t0VTV0ZEdfazFDNElQTjlDeFFGa09MNHRlTU1jcGVZUDZ2al8xMW54UmVNc0E0UFB5ckd5N0Nkb1B1Ynh2a1FxRVQ5YnM5UUJ4Zl9DTU5aanl3U05G?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOaUFhMGUxRXNPeDVmVjV2ajd5Y0VEMHQ3X3E1QVdkLWZYMnpOSjdqX281SjdCYmhkdXpRc1hSRXVoSkdweWs5OXVNa1NENHNpdWVWS25falJkM2FfcC1fUGR3alJKQ0R0QlU4eTFwZ0RVcVFFV1RqWkl5ZWNoV1dYZG1OeGRuZ05JUE11Q2ZjeHVhck8wRzFROFRHdGZIM0VKQ1Ytc2N0a0w0S0QzZlVEMWlnckVTRXFSQmNxZk8xU01NbDBnTE5OUUlIaU9KNFdBT3dPWW5Kb0lxdnZhX1RtR1REeWk2VG5qSDlyUDdrRFVtWHM?oc=5</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>ABC7 Chicago</t>
+          <t>PGA Tour</t>
         </is>
       </c>
       <c r="O50" s="2" t="b">
@@ -4007,31 +4007,31 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 21:01:48</t>
+          <t>2026-08-17 03:20:18</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Applied Materials</t>
+          <t>Deere &amp; Company</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Midday Fly By: Applied Materials reports Q3 beat, Trump slaps tariffs on drones</t>
+          <t>Abelardo de la Espriella asks Donald Trump to suspend tariffs to help Colombia earthquake recovery</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>午間飛行：應用材料公司報告第三季業績超預期，川普對無人機徵收關稅</t>
+          <t>阿韋拉多·德拉埃斯普里埃拉要求唐納德·特朗普暫停關稅以幫助哥倫比亞地震恢復</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>-0.802</v>
+        <v>-0.8080000000000001</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
@@ -4063,12 +4063,12 @@
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQYjlKckVuU2pDZ1RTQXl1MG1WM2lzVWpJVV82U1NaaUZMaWpmRWJMdDVaZ055UUhmNUp3Rm1KMjV4SjVMYS1sVjRDNC1VVmNNNUZGcjAzRk5ZQlM0RGtaNUU5emNfSUxUVmZHZmlkeV9OMHFtX2dZQTR0ZHdqZkx0aEdxOXI3UFlGdXBvMHBQVEhFck92UFJWSUViaHVsTW5XSmJ2NzQ2MXFJaHQ5M0VWWjEzSDQzU29uSWFpeTJlM0h6aTItOFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNVXhoZm85Q3Y5NklZRk8tUUJ6OGc3M2FNOWE0Z1pYWENfdmZVT0FUQ0h4SEJYcWc5THJjRjh3bW1xczhERElnNXpUVko0eEVZLVRLcWkwaTFDX3NBNGl2T1BnYldKVlFoZzltSlMyalVmMEJ2YmRrM19NN0lNQmZBNVp5THl1NERLT1BsMnA5ZXNkTXJUQlpReS1aNE5FXzQ0TVFqUTlsUzNaX0xMM0JsQzVlTkdvNE5OWW9Lb3NNcWJUNG9XSkJvM0xWd9IB0AFBVV95cUxQMU5vNHRDdjVYMEhQQnVvNVRPVTdZVmdBRm1zalNuYmlaSURqckF1NU5PVl9zV0ZSYngweG5KdjFaY25LekVYajFEWDZlQk01V2xTc0FkcGlnSGZWaXpjcV9hNkpzcndHSEZTNGtHTzJzZy0tN0pFYi1XM2t0VTV0ZEdfazFDNElQTjlDeFFGa09MNHRlTU1jcGVZUDZ2al8xMW54UmVNc0E0UFB5ckd5N0Nkb1B1Ynh2a1FxRVQ5YnM5UUJ4Zl9DTU5aanl3U05G?oc=5</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>TipRanks</t>
+          <t>ABC7 Chicago</t>
         </is>
       </c>
       <c r="O51" s="2" t="b">
@@ -4078,31 +4078,31 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 19:00:49</t>
+          <t>2026-08-16 21:01:48</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>DOW</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Dow Inc.</t>
+          <t>Applied Materials</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Dow Drops 1,400 As US Stocks Lead Worldwide Sell-off After Trump's Tariffs Ignite A COVID-like Shock Emergenza (Yzke2pt3Ur)</t>
+          <t>Midday Fly By: Applied Materials reports Q3 beat, Trump slaps tariffs on drones</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>川普的關稅引發了類似新冠病毒的衝擊，美國股市引領全球拋售，道瓊斯指數下跌 1,400 點 (Yzke2pt3Ur)</t>
+          <t>午間飛行：應用材料公司報告第三季業績超預期，川普對無人機徵收關稅</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>-0.743</v>
+        <v>-0.802</v>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
@@ -4134,12 +4134,12 @@
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE0xcFFYdGd0Uzlkb3NrbXhhb3JhZVdPdEVEYms4YTdpQjZtQXl5amhPTnVBallNRlB2MWJ5VG5kWVBCWGNKNHk4em1yUURFdENZT2NfWEgxWE1rQnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQYjlKckVuU2pDZ1RTQXl1MG1WM2lzVWpJVV82U1NaaUZMaWpmRWJMdDVaZ055UUhmNUp3Rm1KMjV4SjVMYS1sVjRDNC1VVmNNNUZGcjAzRk5ZQlM0RGtaNUU5emNfSUxUVmZHZmlkeV9OMHFtX2dZQTR0ZHdqZkx0aEdxOXI3UFlGdXBvMHBQVEhFck92UFJWSUViaHVsTW5XSmJ2NzQ2MXFJaHQ5M0VWWjEzSDQzU29uSWFpeTJlM0h6aTItOFE?oc=5</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>Mshale</t>
+          <t>TipRanks</t>
         </is>
       </c>
       <c r="O52" s="2" t="b">
@@ -4149,31 +4149,31 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 18:59:20</t>
+          <t>2026-08-16 19:00:49</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>DOW</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>General Motors</t>
+          <t>Dow Inc.</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Ford Seeks Tariffs on GM's Korean Imports</t>
+          <t>Dow Drops 1,400 As US Stocks Lead Worldwide Sell-off After Trump's Tariffs Ignite A COVID-like Shock Emergenza (Yzke2pt3Ur)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>福特尋求對通用汽車的韓國進口產品徵收關稅</t>
+          <t>川普的關稅引發了類似新冠病毒的衝擊，美國股市引領全球拋售，道瓊斯指數下跌 1,400 點 (Yzke2pt3Ur)</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>-0.137</v>
+        <v>-0.743</v>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
@@ -4205,12 +4205,12 @@
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPaTR4dU1jOWp5RVJjVXhEY1NvckVYZWFIbXJ1X093ZUd2Z3dNSXUxSW93N2pPQW5NVXhENHpHQnJuSWhJTWdzeEFSa0tpUUNVR2NIVlB2aGtibGozNEY1S1RZdkR0dnZDZnFxQmdhZDdVc1htRGZCUmNEYmpaRkZOSWJpN3p1cG5F?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE0xcFFYdGd0Uzlkb3NrbXhhb3JhZVdPdEVEYms4YTdpQjZtQXl5amhPTnVBallNRlB2MWJ5VG5kWVBCWGNKNHk4em1yUURFdENZT2NfWEgxWE1rQnc?oc=5</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>조선일보</t>
+          <t>Mshale</t>
         </is>
       </c>
       <c r="O53" s="2" t="b">
@@ -4220,45 +4220,45 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 18:50:00</t>
+          <t>2026-08-16 18:59:20</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>RTX Corporation</t>
+          <t>General Motors</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Thieves swap RTX 5080 GPUs for RTX 3060s in Chinese gaming hotels — rogue 'downgrades' go unnoticed until sudden blackout exposes $12,000 heist</t>
+          <t>Ford Seeks Tariffs on GM's Korean Imports</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>竊賊在中國遊戲酒店將 RTX 5080 GPU 換成 RTX 3060——流氓「降級」行為未被注意到，直到突然停電暴露了 12,000 美元的盜竊案</t>
+          <t>福特尋求對通用汽車的韓國進口產品徵收關稅</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>-0.884</v>
+        <v>-0.137</v>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>MARKET</t>
+          <t>GEOPOLITICAL</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>ANALYST_DOWNGRADE</t>
+          <t>TARIFF</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>分析師降評</t>
+          <t>關稅</t>
         </is>
       </c>
       <c r="J54" s="2" t="n">
@@ -4271,17 +4271,17 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>downgrade</t>
+          <t>tariff</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAJBVV95cUxNdXdMS0tYNS0xRjk1N3JCMm9hQ2k2aWZhUkFqVjdHR3NjZ0hKc3paVnh1U2ZtX3VWRDhIY3FnNk8yR3B2TXZiaVpKS0ljczBuNkEzMm9MV01GNUN6cjZDUEVIcWtEb00tQWdlNGpZcmJHdGwzRUpwU3JBS0VPLWgxT0pKNThpNUwxTWplNVNzcGtBaG1XWWhHNnp2SnVqVzlxWkNVaW50SjR6VkV2ai1YbEVqc1dyT0hiSUNCRXI1UXNjTDItN3Z6VXlBZnI3eGE4WWFWMVpVVE1mWmMyZG5xdVpPaG9NQzBkWFBTcGgxZ3ZLQ3lUZG1IZEgyazdBRU1GWTNzX2JEd25zVlNtX3dzdmNTd1FWVE5K?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPaTR4dU1jOWp5RVJjVXhEY1NvckVYZWFIbXJ1X093ZUd2Z3dNSXUxSW93N2pPQW5NVXhENHpHQnJuSWhJTWdzeEFSa0tpUUNVR2NIVlB2aGtibGozNEY1S1RZdkR0dnZDZnFxQmdhZDdVc1htRGZCUmNEYmpaRkZOSWJpN3p1cG5F?oc=5</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>Tom's Hardware</t>
+          <t>조선일보</t>
         </is>
       </c>
       <c r="O54" s="2" t="b">
@@ -4291,49 +4291,49 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:51:44</t>
+          <t>2026-08-16 18:50:00</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Cencora</t>
+          <t>RTX Corporation</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>LOOK: Some areas in Manila are experiencing gutter-deep flooding amid moderate to heavy rains and strong winds as of 8:00 am this Monday, Aug. 17. Affected areas: - Mabini Street cor. Pedro Gil - Gutter Deep - Mabini Street cor. Arsenio Herrera - Gutter De</t>
+          <t>Thieves swap RTX 5080 GPUs for RTX 3060s in Chinese gaming hotels — rogue 'downgrades' go unnoticed until sudden blackout exposes $12,000 heist</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>請注意：截至 8 月 17 日星期一上午 8:00，馬尼拉的一些地區正在經歷中度到大雨和強風的洪水。受影響的地區： - Mabini Street cor.佩德羅·吉爾 - 深溝 - 馬比尼街 Cor。阿塞尼奧·埃雷拉 - Gutter De</t>
+          <t>竊賊在中國遊戲酒店將 RTX 5080 GPU 換成 RTX 3060——流氓「降級」行為未被注意到，直到突然停電暴露了 12,000 美元的盜竊案</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>-0.861</v>
+        <v>-0.884</v>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>OPERATIONS</t>
+          <t>MARKET</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>NATURAL_DISASTER</t>
+          <t>ANALYST_DOWNGRADE</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>天災</t>
+          <t>分析師降評</t>
         </is>
       </c>
       <c r="J55" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
@@ -4342,17 +4342,17 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>flood；flooding</t>
+          <t>downgrade</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNNVQ3a3pCZFFfS0hxZ250cHB4ZGtZaXFrU1RnNFBQTVVzX0JBT19PeDc0dXh1bmFkSWJNbDNRa2h5VlB6XzkydVkxSk9vb3NaNlktYVVTX1J3VlBvLU5rUDVkdXBQMVM1TUxFYlV0UjBVOXdONTN6LXF6RVVzV0x0aExKMUxMTThRSld3V3hqNWpsNW9jS2NNYzcwaVJFaXlTbVhTcE1zU1VfQVo3cnhRX2QyaDllRWFsZm1rQmphMURhMVJGbHlIZ3h4bFhtRDFy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAJBVV95cUxNdXdMS0tYNS0xRjk1N3JCMm9hQ2k2aWZhUkFqVjdHR3NjZ0hKc3paVnh1U2ZtX3VWRDhIY3FnNk8yR3B2TXZiaVpKS0ljczBuNkEzMm9MV01GNUN6cjZDUEVIcWtEb00tQWdlNGpZcmJHdGwzRUpwU3JBS0VPLWgxT0pKNThpNUwxTWplNVNzcGtBaG1XWWhHNnp2SnVqVzlxWkNVaW50SjR6VkV2ai1YbEVqc1dyT0hiSUNCRXI1UXNjTDItN3Z6VXlBZnI3eGE4WWFWMVpVVE1mWmMyZG5xdVpPaG9NQzBkWFBTcGgxZ3ZLQ3lUZG1IZEgyazdBRU1GWTNzX2JEd25zVlNtX3dzdmNTd1FWVE5K?oc=5</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>facebook.com</t>
+          <t>Tom's Hardware</t>
         </is>
       </c>
       <c r="O55" s="2" t="b">
@@ -4362,31 +4362,31 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:44:13</t>
+          <t>2026-08-17 08:51:44</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Lowe's</t>
+          <t>Cencora</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Water level of Danube River approaches record-low due to severe drought</t>
+          <t>LOOK: Some areas in Manila are experiencing gutter-deep flooding amid moderate to heavy rains and strong winds as of 8:00 am this Monday, Aug. 17. Affected areas: - Mabini Street cor. Pedro Gil - Gutter Deep - Mabini Street cor. Arsenio Herrera - Gutter De</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>嚴重乾旱導致多瑙河水位創歷史新低</t>
+          <t>請注意：截至 8 月 17 日星期一上午 8:00，馬尼拉的一些地區正在經歷中度到大雨和強風的洪水。受影響的地區： - Mabini Street cor.佩德羅·吉爾 - 深溝 - 馬比尼街 Cor。阿塞尼奧·埃雷拉 - Gutter De</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>-0.956</v>
+        <v>-0.861</v>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
@@ -4413,17 +4413,17 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>drought</t>
+          <t>flood；flooding</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE93TTlGVFV1ZmxxUGJrYTJyRFRwNzFGT3hLZWlaNkFJeE5uTmY3dXNjUEJfWHJieHR6NVRHQXpEUHB4U05LcnZCNEhoOTVhUV9rYmdzakk3elFGTlY1MHVYSi1LMk1pNFN0YjR2U2JrOFhLUHN3VU1pM3BZTmQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNNVQ3a3pCZFFfS0hxZ250cHB4ZGtZaXFrU1RnNFBQTVVzX0JBT19PeDc0dXh1bmFkSWJNbDNRa2h5VlB6XzkydVkxSk9vb3NaNlktYVVTX1J3VlBvLU5rUDVkdXBQMVM1TUxFYlV0UjBVOXdONTN6LXF6RVVzV0x0aExKMUxMTThRSld3V3hqNWpsNW9jS2NNYzcwaVJFaXlTbVhTcE1zU1VfQVo3cnhRX2QyaDllRWFsZm1rQmphMURhMVJGbHlIZ3h4bFhtRDFy?oc=5</t>
         </is>
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>Xinhua</t>
+          <t>facebook.com</t>
         </is>
       </c>
       <c r="O56" s="2" t="b">
@@ -4433,7 +4433,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:44:12</t>
+          <t>2026-08-17 08:44:13</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -4448,16 +4448,16 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Water level of Danube River approaches record-low due to severe drought-Xinhua</t>
+          <t>Water level of Danube River approaches record-low due to severe drought</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>受嚴重乾旱影響，多瑙河水位創歷史新低-新華社</t>
+          <t>嚴重乾旱導致多瑙河水位創歷史新低</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>-0.902</v>
+        <v>-0.956</v>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
@@ -4489,12 +4489,12 @@
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOcHB0ckl2ZmwtekRfSkVjakJNbVBQNkVQMGkzN0tkdUNINVJiVmZ3OENTbG4xT2dQRjFWS1l1LVRzZjk2N2l0cUR6VUt5SzYxS3pzc3otSXd2aW9lNENSVWRpbFMyVXhWWjk0WmlTWlJwNXRQLWI3VDIzRlhTM1lIdWV3X3JFZFcxbUpVM1owbFBTUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE93TTlGVFV1ZmxxUGJrYTJyRFRwNzFGT3hLZWlaNkFJeE5uTmY3dXNjUEJfWHJieHR6NVRHQXpEUHB4U05LcnZCNEhoOTVhUV9rYmdzakk3elFGTlY1MHVYSi1LMk1pNFN0YjR2U2JrOFhLUHN3VU1pM3BZTmQ?oc=5</t>
         </is>
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>新华网</t>
+          <t>Xinhua</t>
         </is>
       </c>
       <c r="O57" s="2" t="b">
@@ -4504,31 +4504,31 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:23:00</t>
+          <t>2026-08-17 08:44:12</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>LH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Labcorp</t>
+          <t>Lowe's</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>LH mandates elevator air conditioners and boosts flood safety in South Korea - CHOSUNBIZ</t>
+          <t>Water level of Danube River approaches record-low due to severe drought-Xinhua</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>LH 在韓國強制使用電梯空調並提高防洪安全 - CHOSUNBIZ</t>
+          <t>受嚴重乾旱影響，多瑙河水位創歷史新低-新華社</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0.716</v>
+        <v>-0.902</v>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
@@ -4555,17 +4555,17 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>flood</t>
+          <t>drought</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOM1JqUGRwTnpFX25ZWmZGVkstRFp3WEV0b1hvclFGTGwtZ0lMc05JRTJ5UVJDblQxTV96Nl9QNjQ4LVBQM0I0N3AzYVlsZm0xRUoxLXB2RFhMNHBkV1dDTWRVX1lxQ3JJMUpXTjZtdC13V2dQR2oxbXEtcHFJT3dPdWdDYmtTZWhnaThjeVY5eWRiSXJQQXF4QtIBmAFBVV95cUxOM1JqUGRwTnpFX25ZWmZGVkstRFp3WEV0b1hvclFGTGwtZ0lMc05JRTJ5UVJDblQxTV96Nl9QNjQ4LVBQM0I0N3AzYVlsZm0xRUoxLXB2RFhMNHBkV1dDTWRVX1lxQ3JJMUpXTjZtdC13V2dQR2oxbXEtcHFJT3dPdWdDYmtTZWhnaThjeVY5eWRiSXJQQXF4Qg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOcHB0ckl2ZmwtekRfSkVjakJNbVBQNkVQMGkzN0tkdUNINVJiVmZ3OENTbG4xT2dQRjFWS1l1LVRzZjk2N2l0cUR6VUt5SzYxS3pzc3otSXd2aW9lNENSVWRpbFMyVXhWWjk0WmlTWlJwNXRQLWI3VDIzRlhTM1lIdWV3X3JFZFcxbUpVM1owbFBTUQ?oc=5</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>Chosunbiz</t>
+          <t>新华网</t>
         </is>
       </c>
       <c r="O58" s="2" t="b">
@@ -4575,31 +4575,31 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:15:06</t>
+          <t>2026-08-17 08:23:00</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>LH</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Medtronic</t>
+          <t>Labcorp</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Flash Flood Warning in Teller County Remains in Effect Until 8:30 PM MDT</t>
+          <t>LH mandates elevator air conditioners and boosts flood safety in South Korea - CHOSUNBIZ</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>特勒縣山洪預警持續有效，直至太平洋標準時間晚上 8:30</t>
+          <t>LH 在韓國強制使用電梯空調並提高防洪安全 - CHOSUNBIZ</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>-0.458</v>
+        <v>0.716</v>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
@@ -4631,12 +4631,12 @@
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9SWW44bmxPZm9JQTRZeGJXUTd0ZHBVN2xXWllnYkZTVmRUcG9NX0h5amhJLWdOaXRDWVZpTk82WWRzc2p1N3VtQnVLU3daTThPa2g2YmdnZzZkQ1RZZl9Gekd3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOM1JqUGRwTnpFX25ZWmZGVkstRFp3WEV0b1hvclFGTGwtZ0lMc05JRTJ5UVJDblQxTV96Nl9QNjQ4LVBQM0I0N3AzYVlsZm0xRUoxLXB2RFhMNHBkV1dDTWRVX1lxQ3JJMUpXTjZtdC13V2dQR2oxbXEtcHFJT3dPdWdDYmtTZWhnaThjeVY5eWRiSXJQQXF4QtIBmAFBVV95cUxOM1JqUGRwTnpFX25ZWmZGVkstRFp3WEV0b1hvclFGTGwtZ0lMc05JRTJ5UVJDblQxTV96Nl9QNjQ4LVBQM0I0N3AzYVlsZm0xRUoxLXB2RFhMNHBkV1dDTWRVX1lxQ3JJMUpXTjZtdC13V2dQR2oxbXEtcHFJT3dPdWdDYmtTZWhnaThjeVY5eWRiSXJQQXF4Qg?oc=5</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>Forth.News</t>
+          <t>Chosunbiz</t>
         </is>
       </c>
       <c r="O59" s="2" t="b">
@@ -4646,45 +4646,45 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:15:00</t>
+          <t>2026-08-17 08:15:06</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>MDT</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Corning Inc.</t>
+          <t>Medtronic</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Corning (GLW) Stock Looks Overvalued As Its 3 Year Gain Hit 4.5x</t>
+          <t>Flash Flood Warning in Teller County Remains in Effect Until 8:30 PM MDT</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>康寧 (GLW) 股票 3 年漲幅達 4.5 倍，看起來估值過高</t>
+          <t>特勒縣山洪預警持續有效，直至太平洋標準時間晚上 8:30</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.891</v>
+        <v>-0.458</v>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>MARKET</t>
+          <t>OPERATIONS</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>VALUATION_CONCERN</t>
+          <t>NATURAL_DISASTER</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>估值疑慮</t>
+          <t>天災</t>
         </is>
       </c>
       <c r="J60" s="2" t="n">
@@ -4697,17 +4697,17 @@
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>overvalued</t>
+          <t>flood</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxONHd3aVNkT2ZuSWVvOE9fdXZkSTRXN3VyQ21lWS1pcHdjWXUwN2JYbEROa19GUWx0bjh1azJDS0NySzBOcmFQZ0NqSjJpTU9OUmhVdGRWUlpydGYxbS1NSFpWN1JGWk1EeFRwQUEzWG1ITmpDNGtPY0YzWEE5SWtybVVRVFRtdWhnLU9KR0FmSHBqZmJWX3Mxbk9uTmkyU2pk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9SWW44bmxPZm9JQTRZeGJXUTd0ZHBVN2xXWllnYkZTVmRUcG9NX0h5amhJLWdOaXRDWVZpTk82WWRzc2p1N3VtQnVLU3daTThPa2g2YmdnZzZkQ1RZZl9Gekd3?oc=5</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Forth.News</t>
         </is>
       </c>
       <c r="O60" s="2" t="b">
@@ -4717,45 +4717,45 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 08:14:38</t>
+          <t>2026-08-17 08:15:00</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Cencora</t>
+          <t>Corning Inc.</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Moderate to heavy rain with strong winds are currently affecting parts of Manila as of 7:18 a.m., Aug. 17, 2026, according to the Manila DRRM. Gutter-deep flooding reported along: • Quirino Ave. (Vito Cruz) • Quirino Ave. cor. Taft Ave. • Quirino Ave. SB • Padre</t>
+          <t>Corning (GLW) Stock Looks Overvalued As Its 3 Year Gain Hit 4.5x</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>據馬尼拉 DRRM 稱，截至 2026 年 8 月 17 日上午 7 點 18 分，中到大雨和強風目前正在影響馬尼拉部分地區。沿線報告了排水溝深度洪水： • Quirino Ave. (Vito Cruz) • Quirino Ave. cor. (Vito Cruz)塔夫脫大街 • Quirino 大街 SB • Padre</t>
+          <t>康寧 (GLW) 股票 3 年漲幅達 4.5 倍，看起來估值過高</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>-0.735</v>
+        <v>0.891</v>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>OPERATIONS</t>
+          <t>MARKET</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>NATURAL_DISASTER</t>
+          <t>VALUATION_CONCERN</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>天災</t>
+          <t>估值疑慮</t>
         </is>
       </c>
       <c r="J61" s="2" t="n">
@@ -4768,17 +4768,17 @@
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>flood；flooding</t>
+          <t>overvalued</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE4wNFpCZ1VzX1J4M2t1WUpZS0s5dlIwT3pCWVk5UUs1T01BWWdpaFctWUtZNnNRXzdkcU5KdkdPSHRORDA4aTEwektEUWpuWUxXYzBINkxqS3puZEdKQnFYUlpYRXZDWW9Fb0hxSw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxONHd3aVNkT2ZuSWVvOE9fdXZkSTRXN3VyQ21lWS1pcHdjWXUwN2JYbEROa19GUWx0bjh1azJDS0NySzBOcmFQZ0NqSjJpTU9OUmhVdGRWUlpydGYxbS1NSFpWN1JGWk1EeFRwQUEzWG1ITmpDNGtPY0YzWEE5SWtybVVRVFRtdWhnLU9KR0FmSHBqZmJWX3Mxbk9uTmkyU2pk?oc=5</t>
         </is>
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>facebook.com</t>
+          <t>Yahoo Finance</t>
         </is>
       </c>
       <c r="O61" s="2" t="b">
@@ -4788,31 +4788,31 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 07:57:43</t>
+          <t>2026-08-17 08:14:38</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>ServiceNow</t>
+          <t>Cencora</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Active weather now, flash flooding and severe threat remains but a couple days of drier weather awaits</t>
+          <t>Moderate to heavy rain with strong winds are currently affecting parts of Manila as of 7:18 a.m., Aug. 17, 2026, according to the Manila DRRM. Gutter-deep flooding reported along: • Quirino Ave. (Vito Cruz) • Quirino Ave. cor. Taft Ave. • Quirino Ave. SB • Padre</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>目前天氣活躍，山洪暴發和嚴重威脅仍然存在，但未來幾天將出現乾燥天氣</t>
+          <t>據馬尼拉 DRRM 稱，截至 2026 年 8 月 17 日上午 7 點 18 分，中到大雨和強風目前正在影響馬尼拉部分地區。沿線報告了排水溝深度洪水： • Quirino Ave. (Vito Cruz) • Quirino Ave. cor. (Vito Cruz)塔夫脫大街 • Quirino 大街 SB • Padre</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>-0.062</v>
+        <v>-0.735</v>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
@@ -4844,12 +4844,12 @@
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPZWtTWUYxQW9hbmQ0dVJncm5EMl9hZ1lUZDVTcXM0MWRWX0dLeERIVWhpeTdhZkxQOHhxZ19LdHJTaUU0VXFWMTVwNHdVeE80ZVJTVzhSZnBiMlBCbW15LVlDZGVnODg4bVZDUEYtVnlqVXZhblRudGc0NHRNMHhQWlJTdWF3a1R2YkE0VnJhb3pGU2dfS0lQZnVxdWdCYXpDbHoxaXRsMzNsS0Vib3lGOXFvQ0pPX1VDUUtj0gHAAUFVX3lxTE83UzRKbFk4RElodkR1eHpYbjRvc3B1SGVYdm01QmNUZzFqdTF0Y045YW5MX2dZQXpUb1pVVmF5bnI4aUVrQm5EX3dPZUQxaFpnWVNjdV9UdHJrbURWUl92YmY0bjRrOEo5SVJLcTJGalhadUNjNmF2ZWdmMnFhRU1UMTAyQ3dRREtqazV4Qk8xZlNpT2sxSWhNNFZlZTdWTGZxb0tZdTZVaGFYeFZHMFV2NnFtaEp5Nzc3NnVhMk8xRg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE4wNFpCZ1VzX1J4M2t1WUpZS0s5dlIwT3pCWVk5UUs1T01BWWdpaFctWUtZNnNRXzdkcU5KdkdPSHRORDA4aTEwektEUWpuWUxXYzBINkxqS3puZEdKQnFYUlpYRXZDWW9Fb0hxSw?oc=5</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>WOAY-TV</t>
+          <t>facebook.com</t>
         </is>
       </c>
       <c r="O62" s="2" t="b">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQWG1qVjQxNkhkbUZFc3pHZDJxa0xHZzVwQlVPVTFZUXpseDlxaDkzZ19GY3YxQkFwUnNQSVRQNmwxUUhjX3dYRG1RYWtYU3NyNEt0MGJEbkVkdm1QNm9xVV96MVg2WXprSlNuYnBtWmJZZEJNU3ZpeEU0QVhuME12TzA4VW1KR2xFQ3NMRXhhVURyWXF6eTh0cnNGTUFUaDdaUmN5dTZnZ9IBpwFBVV95cUxQWG1qVjQxNkhkbUZFc3pHZDJxa0xHZzVwQlVPVTFZUXpseDlxaDkzZ19GY3YxQkFwUnNQSVRQNmwxUUhjX3dYRG1RYWtYU3NyNEt0MGJEbkVkdm1QNm9xVV96MVg2WXprSlNuYnBtWmJZZEJNU3ZpeEU0QVhuME12TzA4VW1KR2xFQ3NMRXhhVURyWXF6eTh0cnNGTUFUaDdaUmN5dTZnZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNaVp4emlkMmhRRm1qbGI3VjFjTzJaTjgxNDVzRy1SaWh5VFlJdjRGb0FtNHBUQS15VnlzRFdmeDBhVmZKbWRDNVBEdF9QT3BTbGxsUTUyNlRIMjdkZFp5Qm9ORktpVkZudVZDNTJCTk9oaXFMcG9OS3FPSllHaTkydGJmVFhiemZkajVXMktBSzhyeHBkSTNWdjgtQ0pnSklMSG44?oc=5</t>
         </is>
       </c>
       <c r="N74" s="2" t="inlineStr">
@@ -6208,31 +6208,31 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 23:45:00</t>
+          <t>2026-08-16 23:27:57</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Caterpillar Inc.</t>
+          <t>Regency Centers</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Nevada woman flees wildfire with dog, cat, and chickens as pet tegu Noodles escapes</t>
+          <t>NPP Reg. Executive elections: Incumbent Bukari secures landslide mandate, vows 2028 unity victory</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>內華達州婦女帶著狗、貓和雞逃離野火，寵物泰古麵條逃脫</t>
+          <t>核電廠註冊行政選舉：現任布卡里獲得壓倒性授權，誓言 2028 年團結勝利</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>-0.04</v>
+        <v>0.6</v>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
@@ -6259,17 +6259,17 @@
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>wildfire</t>
+          <t>landslide</t>
         </is>
       </c>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNNFlJRm1fZHZHRWFSSG5haTRrcHFfT1l6QUYxMlc3TTRtQTVGMzQ1MTYxai1oa3ZzcHp5TVhzblZISllPMGhlWlk0aFUyZlJBaEI4UHF0dEV0MFFkTXhyalJhamdXbTBVQkxiT1JpUExBamZQZ29OVEh3WG5SRlFKaEZYYkJEa0tuOWJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1CTV9KdFR5Njd5NVJVWTE3b04xS2NPSk0ydWltaEt3X29kU3lmZkJXRWxYVGtacEs1UzhGWklUcHFlZ0RDb2lpdmFOWW9ZYl9DaEJtUmFLcElmbTRqaTA2Mk1EM2TSAVxBVV95cUxQWmJ3b1U2MmZLZ1RTYVF4R2FDLVJsTVZJc2tqdkt6UmFMTjZhTFJiaURQM2RZMngyX1UwVkdSOGxmdS1HSzhlaVcxQk1jeWROeEFISzlmYWlkVmJPZw?oc=5</t>
         </is>
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>The Cool Down</t>
+          <t>modernghana.com</t>
         </is>
       </c>
       <c r="O82" s="2" t="b">
@@ -6279,45 +6279,45 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 23:27:57</t>
+          <t>2026-08-16 23:06:44</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Regency Centers</t>
+          <t>Apple Inc.</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>NPP Reg. Executive elections: Incumbent Bukari secures landslide mandate, vows 2028 unity victory</t>
+          <t>AAPL Looks 8.0% Overvalued on GF Value™ as Guru and Insider Acti</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>核電廠註冊行政選舉：現任布卡里獲得壓倒性授權，誓言 2028 年團結勝利</t>
+          <t>根據 GF Value™ 作為 Guru 和 Insider Acti 的數據，AAPL 的估值被高估了 8.0%</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>0.6</v>
+        <v>-0.19</v>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>OPERATIONS</t>
+          <t>MARKET</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>NATURAL_DISASTER</t>
+          <t>VALUATION_CONCERN</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>天災</t>
+          <t>估值疑慮</t>
         </is>
       </c>
       <c r="J83" s="2" t="n">
@@ -6330,17 +6330,17 @@
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>landslide</t>
+          <t>overvalued</t>
         </is>
       </c>
       <c r="M83" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1CTV9KdFR5Njd5NVJVWTE3b04xS2NPSk0ydWltaEt3X29kU3lmZkJXRWxYVGtacEs1UzhGWklUcHFlZ0RDb2lpdmFOWW9ZYl9DaEJtUmFLcElmbTRqaTA2Mk1EM2TSAVxBVV95cUxQWmJ3b1U2MmZLZ1RTYVF4R2FDLVJsTVZJc2tqdkt6UmFMTjZhTFJiaURQM2RZMngyX1UwVkdSOGxmdS1HSzhlaVcxQk1jeWROeEFISzlmYWlkVmJPZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQbXdhOFgtcWszQ0xpMlZwU3ZLd1FhWXZMRG00NjRwM2pzc1dacHdqMll0RzAtTWIyVmgtMkxIYWZfMjlwbXhlTjhraE5XR1pWTkFYajh6OFU3YkZuZFlGUnVCMS1iQk1fRmxpMU5vd1VIeHJ0RmJBaTItMEFyNjZVUXJfNVJfaS1NZFNkaGlVTkVXaHpIbW0tXy1PbU1UY2pXSnRucldaN2FBQzl3Sng0R21ZRzFsdlI0bmZNQw?oc=5</t>
         </is>
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>modernghana.com</t>
+          <t>GuruFocus</t>
         </is>
       </c>
       <c r="O83" s="2" t="b">
@@ -6355,26 +6355,26 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Apple Inc.</t>
+          <t>Delta Air Lines</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>AAPL Looks 8.0% Overvalued on GF Value™ as Guru and Insider Acti</t>
+          <t>DAL Looks 51.4% Overvalued on GF Value™ as Direct Austin-Paris F</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>根據 GF Value™ 作為 Guru 和 Insider Acti 的數據，AAPL 的估值被高估了 8.0%</t>
+          <t>DAL 在 GF Value™ 上看起來被高估了 51.4%，因為直接奧斯汀-巴黎 F</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>-0.19</v>
+        <v>0.627</v>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQbXdhOFgtcWszQ0xpMlZwU3ZLd1FhWXZMRG00NjRwM2pzc1dacHdqMll0RzAtTWIyVmgtMkxIYWZfMjlwbXhlTjhraE5XR1pWTkFYajh6OFU3YkZuZFlGUnVCMS1iQk1fRmxpMU5vd1VIeHJ0RmJBaTItMEFyNjZVUXJfNVJfaS1NZFNkaGlVTkVXaHpIbW0tXy1PbU1UY2pXSnRucldaN2FBQzl3Sng0R21ZRzFsdlI0bmZNQw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVGtWajZ6ODVLZzlRaU9Ya2dZbnZTWWZTeUhPMUhZSVNlaFMxS3J6Z243ay1IM3BRRjZXNWVBR0Y0bWN4RXlVNUt2MXVIU0pvQi1WUWhIbTlqUXpweHA1enVKYnlTOE93N2hleExvMi0xeUtQY0FvYUNOTlNRZWRCVDJ6MFRvSnJQNUg2Um14amFZYWRFeXZyTXRXWldKZTNTZ2pwR2xxWVhtM2VNOHB6OTVZaThwZw?oc=5</t>
         </is>
       </c>
       <c r="N84" s="2" t="inlineStr">
@@ -6421,45 +6421,45 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 23:06:44</t>
+          <t>2026-08-16 23:00:00</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>V</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Delta Air Lines</t>
+          <t>Visa Inc.</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>DAL Looks 51.4% Overvalued on GF Value™ as Direct Austin-Paris F</t>
+          <t>San Jose Earthquakes v Minnesota Utd Odds</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>DAL 在 GF Value™ 上看起來被高估了 51.4%，因為直接奧斯汀-巴黎 F</t>
+          <t>聖荷西地震 v 明尼蘇達聯隊 賠率</t>
         </is>
       </c>
       <c r="F85" s="2" t="n">
-        <v>0.627</v>
+        <v>0.023</v>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>MARKET</t>
+          <t>OPERATIONS</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>VALUATION_CONCERN</t>
+          <t>NATURAL_DISASTER</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>估值疑慮</t>
+          <t>天災</t>
         </is>
       </c>
       <c r="J85" s="2" t="n">
@@ -6472,17 +6472,17 @@
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>overvalued</t>
+          <t>earthquake</t>
         </is>
       </c>
       <c r="M85" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVGtWajZ6ODVLZzlRaU9Ya2dZbnZTWWZTeUhPMUhZSVNlaFMxS3J6Z243ay1IM3BRRjZXNWVBR0Y0bWN4RXlVNUt2MXVIU0pvQi1WUWhIbTlqUXpweHA1enVKYnlTOE93N2hleExvMi0xeUtQY0FvYUNOTlNRZWRCVDJ6MFRvSnJQNUg2Um14amFZYWRFeXZyTXRXWldKZTNTZ2pwR2xxWVhtM2VNOHB6OTVZaThwZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQMlA0R0RKTHlFbW0tZ043eUlvb2lOOGE4eDRXN2FMaGV6Y3htYmt0a25kV1BuTTh3ODNpM2p5bTl4c3NaQ2dBeDYzU0d5dHpCdm1HT3RncjJPNFh3bXJPWnJabDd6YkhJOTNLWDdpd0JVTUQ2RV9LYWtObmZ3cUJQU1d0Tmlqc2JCSjZpMHRmd2t6a3BR?oc=5</t>
         </is>
       </c>
       <c r="N85" s="2" t="inlineStr">
         <is>
-          <t>GuruFocus</t>
+          <t>FanDuel Sportsbook</t>
         </is>
       </c>
       <c r="O85" s="2" t="b">
@@ -6492,45 +6492,45 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 23:00:00</t>
+          <t>2026-08-16 22:48:27</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Visa Inc.</t>
+          <t>Apple Inc.</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>San Jose Earthquakes v Minnesota Utd Odds</t>
+          <t>AAPL Looks 8.0% Overvalued on GF Value™ as Insider Selling Persi</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>聖荷西地震 v 明尼蘇達聯隊 賠率</t>
+          <t>由於內線交易 Persi，GF Value™ 使 AAPL 的估值被高估了 8.0%</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>0.023</v>
+        <v>-0.748</v>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>OPERATIONS</t>
+          <t>MARKET</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>NATURAL_DISASTER</t>
+          <t>VALUATION_CONCERN</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>天災</t>
+          <t>估值疑慮</t>
         </is>
       </c>
       <c r="J86" s="2" t="n">
@@ -6543,17 +6543,17 @@
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>earthquake</t>
+          <t>overvalued</t>
         </is>
       </c>
       <c r="M86" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQMlA0R0RKTHlFbW0tZ043eUlvb2lOOGE4eDRXN2FMaGV6Y3htYmt0a25kV1BuTTh3ODNpM2p5bTl4c3NaQ2dBeDYzU0d5dHpCdm1HT3RncjJPNFh3bXJPWnJabDd6YkhJOTNLWDdpd0JVTUQ2RV9LYWtObmZ3cUJQU1d0Tmlqc2JCSjZpMHRmd2t6a3BR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNT0hEVU1RZmV4Yk1BaEZiZkpqX0huUmdWc1JKSEFtekdKT1VRVW0teWRNOFN5ZnFIdzBaRWVpSU5paFg3MXpBTVp6dXVmQ05SYmtkamlEZG10N01WdHE0ZW5zTkxDY0Jkb0VtcEdPZE9sV2lSWVNXWTEwWXJwRjYxZGV0aXZTMDgxS2VZUE9jcElWUkVoQXcxbWNrMURFTVpITmphdU13?oc=5</t>
         </is>
       </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>FanDuel Sportsbook</t>
+          <t>GuruFocus</t>
         </is>
       </c>
       <c r="O86" s="2" t="b">
@@ -6568,26 +6568,26 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Apple Inc.</t>
+          <t>Digital Realty</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>AAPL Looks 8.0% Overvalued on GF Value™ as Insider Selling Persi</t>
+          <t>DLR Looks 67.6% Overvalued on GF Value™ Amid Dividend Sustainabi</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>由於內線交易 Persi，GF Value™ 使 AAPL 的估值被高估了 8.0%</t>
+          <t>在股息可持續發展的情況下，DLR 的 GF Value™ 估值被高估了 67.6%</t>
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>-0.748</v>
+        <v>-0.735</v>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
@@ -6619,7 +6619,7 @@
       </c>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNT0hEVU1RZmV4Yk1BaEZiZkpqX0huUmdWc1JKSEFtekdKT1VRVW0teWRNOFN5ZnFIdzBaRWVpSU5paFg3MXpBTVp6dXVmQ05SYmtkamlEZG10N01WdHE0ZW5zTkxDY0Jkb0VtcEdPZE9sV2lSWVNXWTEwWXJwRjYxZGV0aXZTMDgxS2VZUE9jcElWUkVoQXcxbWNrMURFTVpITmphdU13?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNWmJBMUpMMU5QTUxuSm5nZHlkN21XbEpuQ1dLbmVVczR6NW5wd2htUGxMdmZtQVBVYUllQWJaNHQ3X2pQWmlpU1ZVa0lKMHZaOExyMUtEMUtjUnprU0x6WFotRXJYQjYzV3FfbU5ldlJqNkF2d211anNoZlV3RUVKR21SbzJzVmozZVB6emhpZ0oteEM1cGVlODRkTURaaVhaTmFxNmthbjJzOU91a0ZLWWYxQQ?oc=5</t>
         </is>
       </c>
       <c r="N87" s="2" t="inlineStr">
@@ -6639,26 +6639,26 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Digital Realty</t>
+          <t>Bristol Myers Squibb</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>DLR Looks 67.6% Overvalued on GF Value™ Amid Dividend Sustainabi</t>
+          <t>BMY Looks 13.0% Overvalued on GF Value™ Amid $6.7B Lawsuit Reins</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>在股息可持續發展的情況下，DLR 的 GF Value™ 估值被高估了 67.6%</t>
+          <t>在 $6.7B 訴訟中，BMY 在 GF Value™ 上看起來被高估了 13.0%</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>-0.735</v>
+        <v>-0.68</v>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
@@ -6690,7 +6690,7 @@
       </c>
       <c r="M88" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNWmJBMUpMMU5QTUxuSm5nZHlkN21XbEpuQ1dLbmVVczR6NW5wd2htUGxMdmZtQVBVYUllQWJaNHQ3X2pQWmlpU1ZVa0lKMHZaOExyMUtEMUtjUnprU0x6WFotRXJYQjYzV3FfbU5ldlJqNkF2d211anNoZlV3RUVKR21SbzJzVmozZVB6emhpZ0oteEM1cGVlODRkTURaaVhaTmFxNmthbjJzOU91a0ZLWWYxQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOeHJoNVpoeG5FM3VmWTlPUWhVYl9CQkU4Vzd4TGd1bEJreWhoSVBqN0dncmhzbkJ6c0dBeWgwb0pmNlNJSEUyVGhYT2RUcDR1SlQyamMtT0tPZ1hteUdsODU2TnREV2c4TnM0UjlJSDgtXzVCN2xkNExvSldpYVhZN1cyemlKci12MnZjLXFkblhkWk9CNEhjWXdIc3NBWXJCUlRpcGtZRldTUQ?oc=5</t>
         </is>
       </c>
       <c r="N88" s="2" t="inlineStr">
@@ -6710,26 +6710,26 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Bristol Myers Squibb</t>
+          <t>Applied Materials</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>BMY Looks 13.0% Overvalued on GF Value™ Amid $6.7B Lawsuit Reins</t>
+          <t>AMAT Looks 116.4% Overvalued on GF Value™</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>在 $6.7B 訴訟中，BMY 在 GF Value™ 上看起來被高估了 13.0%</t>
+          <t>GF Value™ 上 AMAT 的估價被高估了 116.4%</t>
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>-0.68</v>
+        <v>0.444</v>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="M89" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOeHJoNVpoeG5FM3VmWTlPUWhVYl9CQkU4Vzd4TGd1bEJreWhoSVBqN0dncmhzbkJ6c0dBeWgwb0pmNlNJSEUyVGhYT2RUcDR1SlQyamMtT0tPZ1hteUdsODU2TnREV2c4TnM0UjlJSDgtXzVCN2xkNExvSldpYVhZN1cyemlKci12MnZjLXFkblhkWk9CNEhjWXdIc3NBWXJCUlRpcGtZRldTUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQd3dHdnp2aTdSeEZ3NUxhQzNGZlFJNUF5QkxGMnAyeDh5YjhzN3NfVkJfTFRkOHIxaVQtdUhtLVBQMWhXS3NkeEtOZ0hFajRkMWRnZmVPNXA1ek8wbE1PZUdXZ2RySFFndGRndmJFOTFITC1BNXVjTVhhZmUzbWp1VkRxZw?oc=5</t>
         </is>
       </c>
       <c r="N89" s="2" t="inlineStr">
@@ -6776,31 +6776,31 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 22:48:27</t>
+          <t>2026-08-16 22:08:22</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Applied Materials</t>
+          <t>Colgate-Palmolive</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>AMAT Looks 116.4% Overvalued on GF Value™</t>
+          <t>Colgate-Palmolive (CL) Could Be 30% Undervalued Despite A 6% Overvalued Narrative</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>GF Value™ 上 AMAT 的估價被高估了 116.4%</t>
+          <t>高露潔棕欖 (CL) 的估值可能被低估 30%，儘管其估值被高估了 6%</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>0.444</v>
+        <v>0.87</v>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
@@ -6832,12 +6832,12 @@
       </c>
       <c r="M90" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQd3dHdnp2aTdSeEZ3NUxhQzNGZlFJNUF5QkxGMnAyeDh5YjhzN3NfVkJfTFRkOHIxaVQtdUhtLVBQMWhXS3NkeEtOZ0hFajRkMWRnZmVPNXA1ek8wbE1PZUdXZ2RySFFndGRndmJFOTFITC1BNXVjTVhhZmUzbWp1VkRxZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOOTdEbS1iMVdTVHRsVFE1WGptVk9iNF9WaVlLNXh0SmxjSU9hMEVXMjl1Zkc0T1h1T2hhbDlkT01hbXlGbUd5QWtfcGs3bVAxX2tvWE94X1h3eUVuYUpIMmJjUjhTY2ktZWJnMmYtQmIwYnNSdWViUDAwNUVYQ1RsWEh0TU9ZLUg2WWhYeUFSUWdBYVcxdzdlRGhn?oc=5</t>
         </is>
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>GuruFocus</t>
+          <t>Yahoo Finance</t>
         </is>
       </c>
       <c r="O90" s="2" t="b">
@@ -6847,31 +6847,31 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 22:08:22</t>
+          <t>2026-08-16 22:08:15</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Colgate-Palmolive</t>
+          <t>Hewlett Packard Enterprise</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Colgate-Palmolive (CL) Could Be 30% Undervalued Despite A 6% Overvalued Narrative</t>
+          <t>HPE Looks 132.3% Overvalued on GF Value™ as DOJ Approves Juniper Acquisition</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>高露潔棕欖 (CL) 的估值可能被低估 30%，儘管其估值被高估了 6%</t>
+          <t>隨著美國司法部批准瞻博網路收購，HPE 在 GF Value™ 上的估值被高估了 132.3%</t>
         </is>
       </c>
       <c r="F91" s="2" t="n">
-        <v>0.87</v>
+        <v>0.643</v>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
@@ -6903,12 +6903,12 @@
       </c>
       <c r="M91" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOOTdEbS1iMVdTVHRsVFE1WGptVk9iNF9WaVlLNXh0SmxjSU9hMEVXMjl1Zkc0T1h1T2hhbDlkT01hbXlGbUd5QWtfcGs3bVAxX2tvWE94X1h3eUVuYUpIMmJjUjhTY2ktZWJnMmYtQmIwYnNSdWViUDAwNUVYQ1RsWEh0TU9ZLUg2WWhYeUFSUWdBYVcxdzdlRGhn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxOYTJGTHpUMU1hY1AwcW1OR0JIN09WWVZaWExXeUFneW03VXM2TDMyR2NLeEVEdDd4S0pzVVFNOHJGYzBGYjJmTko0eWpiT0owdDN4OUVXeUxBN2paQ0I2T0lVX1h2elRqeDRnbE9qMGpQcWFLbldhTDdxdTR5LThYYklBODFMVWxXWlVNMkUxS2lCTGJNQXRNSDBabEktU0tEa1NRTFRhcjBvbWlLODUyN093?oc=5</t>
         </is>
       </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>GuruFocus</t>
         </is>
       </c>
       <c r="O91" s="2" t="b">
@@ -6918,31 +6918,31 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 22:08:15</t>
+          <t>2026-08-16 21:39:30</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Hewlett Packard Enterprise</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>HPE Looks 132.3% Overvalued on GF Value™ as DOJ Approves Juniper Acquisition</t>
+          <t>CSCO Looks 55.6% Overvalued on GF Value™</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>隨著美國司法部批准瞻博網路收購，HPE 在 GF Value™ 上的估值被高估了 132.3%</t>
+          <t>GF Value™ 認為 CSCO 被高估了 55.6%</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>0.643</v>
+        <v>0.019</v>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
@@ -6974,7 +6974,7 @@
       </c>
       <c r="M92" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxOYTJGTHpUMU1hY1AwcW1OR0JIN09WWVZaWExXeUFneW03VXM2TDMyR2NLeEVEdDd4S0pzVVFNOHJGYzBGYjJmTko0eWpiT0owdDN4OUVXeUxBN2paQ0I2T0lVX1h2elRqeDRnbE9qMGpQcWFLbldhTDdxdTR5LThYYklBODFMVWxXWlVNMkUxS2lCTGJNQXRNSDBabEktU0tEa1NRTFRhcjBvbWlLODUyN093?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPMFNOWnd4bEhVZkk2dUlfcDFoYnNpdU9HUnhpQ0gwMnk0SWtiVUM4R19UaTh6YjNGaHJ2d0tCU3MteS1YbmN5dkpERlZEMkpmci1DdjRGRWZEdGtwWmhRZmFTM0lSRVFsWGU1dkZhZ1dRN3JURlF2ZkN6MDlEbGZHRkpn?oc=5</t>
         </is>
       </c>
       <c r="N92" s="2" t="inlineStr">
@@ -6989,31 +6989,31 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 21:39:30</t>
+          <t>2026-08-16 21:09:33</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>CSCO Looks 55.6% Overvalued on GF Value™</t>
+          <t>BA Looks 10.1% Overvalued on GF Value™ Amid Contract Expansion</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>GF Value™ 認為 CSCO 被高估了 55.6%</t>
+          <t>在合約擴張期間，BA 的 GF Value™ 估值被高估了 10.1%</t>
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>0.019</v>
+        <v>0.19</v>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
@@ -7045,7 +7045,7 @@
       </c>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPMFNOWnd4bEhVZkk2dUlfcDFoYnNpdU9HUnhpQ0gwMnk0SWtiVUM4R19UaTh6YjNGaHJ2d0tCU3MteS1YbmN5dkpERlZEMkpmci1DdjRGRWZEdGtwWmhRZmFTM0lSRVFsWGU1dkZhZ1dRN3JURlF2ZkN6MDlEbGZHRkpn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOdVNjR3hWR1QybHRuYllobGtJbjhzUE5aZElqQm1ENmtFakt1RnZFZ0VRUGRCTnVQREhoRjBWXy1vdUhXbHFWcUk2UGJibzF5WEdMb0xoQ005U1JiQm9qcFY1YjBNa29OUF9yTWYyb3ROVDlDa3BNS0pnSDUxLWhqbDBtUEtIOXJjSy1DZ0pIOWQtMThKQnIweGdkdFd1Mms?oc=5</t>
         </is>
       </c>
       <c r="N93" s="2" t="inlineStr">
@@ -7060,45 +7060,45 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 21:09:33</t>
+          <t>2026-08-16 20:41:00</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>Estée Lauder Companies (The)</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>BA Looks 10.1% Overvalued on GF Value™ Amid Contract Expansion</t>
+          <t>El Niño keeps Atlantic hurricane activity unusually quiet</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>在合約擴張期間，BA 的 GF Value™ 估值被高估了 10.1%</t>
+          <t>厄爾尼諾現象使大西洋颶風活動異常平靜</t>
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>0.19</v>
+        <v>-0.844</v>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>MARKET</t>
+          <t>OPERATIONS</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>VALUATION_CONCERN</t>
+          <t>NATURAL_DISASTER</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>估值疑慮</t>
+          <t>天災</t>
         </is>
       </c>
       <c r="J94" s="2" t="n">
@@ -7111,17 +7111,17 @@
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>overvalued</t>
+          <t>hurricane</t>
         </is>
       </c>
       <c r="M94" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOdVNjR3hWR1QybHRuYllobGtJbjhzUE5aZElqQm1ENmtFakt1RnZFZ0VRUGRCTnVQREhoRjBWXy1vdUhXbHFWcUk2UGJibzF5WEdMb0xoQ005U1JiQm9qcFY1YjBNa29OUF9yTWYyb3ROVDlDa3BNS0pnSDUxLWhqbDBtUEtIOXJjSy1DZ0pIOWQtMThKQnIweGdkdFd1Mms?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxONUdoVEFFZ0NxZlJYaGp2QzhlWHhORGcybmFrTE5VQWlCaGFDdHpQXzVsU056enZzWHhNbE9USVIwRkhsZmJDUzdlVFZ1R2lCSW1ZeFN0VDJtVzQyc0Y1NHJFa2Izb1ZhSWxRcWFoQUNETXVrUlBsXy1xdTN4NTFkVzRsVEN4bGo3N2ZpaFRhTTN0UFp6?oc=5</t>
         </is>
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>GuruFocus</t>
+          <t>fpren.org</t>
         </is>
       </c>
       <c r="O94" s="2" t="b">
@@ -7131,31 +7131,31 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 20:41:00</t>
+          <t>2026-08-16 20:35:00</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>EL</t>
+          <t>NI</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Estée Lauder Companies (The)</t>
+          <t>NiSource</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>El Niño keeps Atlantic hurricane activity unusually quiet</t>
+          <t>Kagwe assures Kenyans of food security despite drought threat ni</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>厄爾尼諾現象使大西洋颶風活動異常平靜</t>
+          <t>卡格威向肯亞人民保證糧食安全，儘管面臨乾旱威脅</t>
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>-0.844</v>
+        <v>0.772</v>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
@@ -7182,17 +7182,17 @@
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>hurricane</t>
+          <t>drought</t>
         </is>
       </c>
       <c r="M95" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxONUdoVEFFZ0NxZlJYaGp2QzhlWHhORGcybmFrTE5VQWlCaGFDdHpQXzVsU056enZzWHhNbE9USVIwRkhsZmJDUzdlVFZ1R2lCSW1ZeFN0VDJtVzQyc0Y1NHJFa2Izb1ZhSWxRcWFoQUNETXVrUlBsXy1xdTN4NTFkVzRsVEN4bGo3N2ZpaFRhTTN0UFp6?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQNWR1eEhCSmZ6SHJLMjBUN2N2WXB1SzhFcGE1WElNRVdjekc5WjU2NmdVbktTN2NkTVgtVjlBUkNOQzdMaUFoZGc3aWJyZWFPZDVFcmQwc0E5V2RvNWl5REwtQ0lMaWpRQ00wVDdjY01wV1JlSGk3ZEdsYnVGdkZhTmxFZ1VNUlVVVWdFWlVMNGJlSFU2UW9USnJGNzl0QktNeGZFUjFHQQ?oc=5</t>
         </is>
       </c>
       <c r="N95" s="2" t="inlineStr">
         <is>
-          <t>fpren.org</t>
+          <t>the-star.co.ke</t>
         </is>
       </c>
       <c r="O95" s="2" t="b">
@@ -7202,31 +7202,31 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 20:35:00</t>
+          <t>2026-08-16 18:10:56</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>NI</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>NiSource</t>
+          <t>Consolidated Edison</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Kagwe assures Kenyans of food security despite drought threat ni</t>
+          <t>HDOT Director Ed Sniffen gives update on closures, road conditions affected by Hurricane Lala</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>卡格威向肯亞人民保證糧食安全，儘管面臨乾旱威脅</t>
+          <t>HDOT 總監 Ed Sniffen 介紹了受颶風拉拉影響的封閉和路況的最新情況</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>0.772</v>
+        <v>-0.421</v>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
@@ -7253,17 +7253,17 @@
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>drought</t>
+          <t>hurricane</t>
         </is>
       </c>
       <c r="M96" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQNWR1eEhCSmZ6SHJLMjBUN2N2WXB1SzhFcGE1WElNRVdjekc5WjU2NmdVbktTN2NkTVgtVjlBUkNOQzdMaUFoZGc3aWJyZWFPZDVFcmQwc0E5V2RvNWl5REwtQ0lMaWpRQ00wVDdjY01wV1JlSGk3ZEdsYnVGdkZhTmxFZ1VNUlVVVWdFWlVMNGJlSFU2UW9USnJGNzl0QktNeGZFUjFHQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOQUxtVzhINjRUTXY5SzFmMzBfX2g3YUk1QVdDQk5zcjh6bTJNUDF5QklHQ0hwYmU2cmJqVUpIbG1rUkRyaklQeUZURUZkR3JmWWp3RDNoX1dhd2ZOVWFlRXkwenY3TW5PVFRsQzVHcVlBaWpobFpRUDkxQXlTOGNpbWN0aUVhalotYWtaRFliU3dqSGcxMC0zR08tLXI5d2ZYaDFTMkQzYWNTNURMQ3htb3V0UGt5RXBTNDhHSzdzVFJuRkZxUWdJeWVMRlNyRnc5TndN?oc=5</t>
         </is>
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>the-star.co.ke</t>
+          <t>Hawaii News Now</t>
         </is>
       </c>
       <c r="O96" s="2" t="b">
@@ -7273,31 +7273,31 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 18:10:56</t>
+          <t>2026-08-16 17:55:22</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>BRO</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Consolidated Edison</t>
+          <t>Brown &amp; Brown</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>HDOT Director Ed Sniffen gives update on closures, road conditions affected by Hurricane Lala</t>
+          <t>BRO Clears Landslides On Rajouri-Poonch NH-144, Works Round-The-Clock To Restore Connectivity</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>HDOT 總監 Ed Sniffen 介紹了受颶風拉拉影響的封閉和路況的最新情況</t>
+          <t>BRO 清除 Rajouri-Poonch NH-144 山體滑坡，全天候工作以恢復連接</t>
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>-0.421</v>
+        <v>0.279</v>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
@@ -7324,17 +7324,17 @@
       </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t>hurricane</t>
+          <t>landslide</t>
         </is>
       </c>
       <c r="M97" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOQUxtVzhINjRUTXY5SzFmMzBfX2g3YUk1QVdDQk5zcjh6bTJNUDF5QklHQ0hwYmU2cmJqVUpIbG1rUkRyaklQeUZURUZkR3JmWWp3RDNoX1dhd2ZOVWFlRXkwenY3TW5PVFRsQzVHcVlBaWpobFpRUDkxQXlTOGNpbWN0aUVhalotYWtaRFliU3dqSGcxMC0zR08tLXI5d2ZYaDFTMkQzYWNTNURMQ3htb3V0UGt5RXBTNDhHSzdzVFJuRkZxUWdJeWVMRlNyRnc5TndN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPSlBPOUxla1IwV0xtUHFjWm41ZnE3bXJhd19rNGxTa29FcmJHZDhXbU1kRnI3andEWGQ2d3JWTy05VnhrZGVpLWdXbFRzZnR2cHg2Y3FZclhwV01hWFlYdC1YTWdPeTRZU2hDaTVGRmM4aGh2eHkyNzI4QVpTdWxKYlgyUVo2SmN6Yk8tQlRDdUJMeDFvQ2E2YVFiSzFna1JSdnlzbjBPVjFOVUdsOVlwYkhxMEE?oc=5</t>
         </is>
       </c>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>Hawaii News Now</t>
+          <t>earthnews.in</t>
         </is>
       </c>
       <c r="O97" s="2" t="b">
@@ -7344,7 +7344,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 17:55:22</t>
+          <t>2026-08-16 17:39:11</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -7359,16 +7359,16 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>BRO Clears Landslides On Rajouri-Poonch NH-144, Works Round-The-Clock To Restore Connectivity</t>
+          <t>BRO Clears Landslides On Rajouri-Poonch NH-144, Work Round-The-Clock To Restore Connectivity After Flash Floods</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>BRO 清除 Rajouri-Poonch NH-144 山體滑坡，全天候工作以恢復連接</t>
+          <t>BRO 清除 Rajouri-Poonch NH-144 山體滑坡，全天候工作以在山洪暴發後恢復連接</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>0.279</v>
+        <v>0.369</v>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
@@ -7395,17 +7395,17 @@
       </c>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t>landslide</t>
+          <t>flood；landslide</t>
         </is>
       </c>
       <c r="M98" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPSlBPOUxla1IwV0xtUHFjWm41ZnE3bXJhd19rNGxTa29FcmJHZDhXbU1kRnI3andEWGQ2d3JWTy05VnhrZGVpLWdXbFRzZnR2cHg2Y3FZclhwV01hWFlYdC1YTWdPeTRZU2hDaTVGRmM4aGh2eHkyNzI4QVpTdWxKYlgyUVo2SmN6Yk8tQlRDdUJMeDFvQ2E2YVFiSzFna1JSdnlzbjBPVjFOVUdsOVlwYkhxMEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxOcm1OV1M4QlJtMi1mX1psMFpYSm1hNGpQMkwwZWtDdXhVbnNHbjF3WVJ6VS1iVExMT05HbnFyZTVmaF9RRjFVcnNKc05yaXBzTnFFcmlDMTIyR0R3ZW1hd1lCdEw3MVZacjRoT3F3U3FTbWVyT1hIaGJYeEE1a2lMaWNUWWR5RFJyWWtzNEZtcm5wYXJWTDRQSmgyQXBSb1dWV1ZEU21xRzFHWUNwS3FiV0U3SVRsYWpTNkp5ZzZRTXhuYnNsLUpQX1hSZ3JZTV8xek84SFZReTItRi1LNlHSAd4BQVVfeXFMTnJtTldTOEJSbTItZl9abDBaWEptYTRqUDJMMGVrQ3V4VW5zR24xd1lSelUtYlRMTE9OR25xcmU1ZmhfUUYxVXJzSnNOcmlwc05xRXJpQzEyMkdEd2VtYXdZQnRMNzFWWnI0aE9xd1NxU21lck9YSGhiWHhBNWtpTGljVFlkeURScllrczRGbXJucGFyVkw0UEpoMkFwUm9XVldWRFNtcUcxR1lDcEtxYldFN0lUbGFqUzZKeWc2UU14bmJzbC1KUF9YUmdyWU1fMXpPOEhWUXkyLUYtSzZR?oc=5</t>
         </is>
       </c>
       <c r="N98" s="2" t="inlineStr">
         <is>
-          <t>earthnews.in</t>
+          <t>Daily Excelsior</t>
         </is>
       </c>
       <c r="O98" s="2" t="b">
@@ -7415,7 +7415,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 17:39:11</t>
+          <t>2026-08-16 17:12:25</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -7430,16 +7430,16 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>BRO Clears Landslides On Rajouri-Poonch NH-144, Work Round-The-Clock To Restore Connectivity After Flash Floods</t>
+          <t>BRO clears landslides on Rajouri-Poonch NH-144 to restore connectivity</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>BRO 清除 Rajouri-Poonch NH-144 山體滑坡，全天候工作以在山洪暴發後恢復連接</t>
+          <t>BRO 清理了 Rajouri-Poonch NH-144 上的山體滑坡以恢復連通性</t>
         </is>
       </c>
       <c r="F99" s="2" t="n">
-        <v>0.369</v>
+        <v>0.465</v>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
@@ -7466,17 +7466,17 @@
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>flood；landslide</t>
+          <t>landslide</t>
         </is>
       </c>
       <c r="M99" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxOcm1OV1M4QlJtMi1mX1psMFpYSm1hNGpQMkwwZWtDdXhVbnNHbjF3WVJ6VS1iVExMT05HbnFyZTVmaF9RRjFVcnNKc05yaXBzTnFFcmlDMTIyR0R3ZW1hd1lCdEw3MVZacjRoT3F3U3FTbWVyT1hIaGJYeEE1a2lMaWNUWWR5RFJyWWtzNEZtcm5wYXJWTDRQSmgyQXBSb1dWV1ZEU21xRzFHWUNwS3FiV0U3SVRsYWpTNkp5ZzZRTXhuYnNsLUpQX1hSZ3JZTV8xek84SFZReTItRi1LNlHSAd4BQVVfeXFMTnJtTldTOEJSbTItZl9abDBaWEptYTRqUDJMMGVrQ3V4VW5zR24xd1lSelUtYlRMTE9OR25xcmU1ZmhfUUYxVXJzSnNOcmlwc05xRXJpQzEyMkdEd2VtYXdZQnRMNzFWWnI0aE9xd1NxU21lck9YSGhiWHhBNWtpTGljVFlkeURScllrczRGbXJucGFyVkw0UEpoMkFwUm9XVldWRFNtcUcxR1lDcEtxYldFN0lUbGFqUzZKeWc2UU14bmJzbC1KUF9YUmdyWU1fMXpPOEhWUXkyLUYtSzZR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPOGtyZkxLUEMwUE10MWFiLXlEX2lHWm54TU1ldGYzNS1jLWtQRjRHa1FoY3JUMkE4X0dkTmpDV204aWpmUlhVZmFKczZXRGllTE5aWnhPX2xwSE9tWmpzQmlXOVh6dTd2TnJJbWhaSmkyZHdrTzlxT2J3NmpkWmNBZHlzdUpmblVBd1JJS0ZSQlJKa3dqMlZ3cHBNZlozTFoxZ2tMLXB3?oc=5</t>
         </is>
       </c>
       <c r="N99" s="2" t="inlineStr">
         <is>
-          <t>Daily Excelsior</t>
+          <t>The News Mill</t>
         </is>
       </c>
       <c r="O99" s="2" t="b">
@@ -7486,31 +7486,31 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 17:12:25</t>
+          <t>2026-08-16 16:56:17</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>BRO</t>
+          <t>O</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Brown &amp; Brown</t>
+          <t>Realty Income</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>BRO clears landslides on Rajouri-Poonch NH-144 to restore connectivity</t>
+          <t>City urges residents to stay safe as Hurricane Lala passes O‘ahu; TheBus service temporarily suspended due to extreme weather</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>BRO 清理了 Rajouri-Poonch NH-144 上的山體滑坡以恢復連通性</t>
+          <t>颶風拉拉經過歐胡島時，市政府敦促居民保持安全；巴士服務因極端天氣而暫停</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>0.465</v>
+        <v>-0.917</v>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
@@ -7537,96 +7537,25 @@
       </c>
       <c r="L100" s="2" t="inlineStr">
         <is>
-          <t>landslide</t>
+          <t>hurricane</t>
         </is>
       </c>
       <c r="M100" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPOGtyZkxLUEMwUE10MWFiLXlEX2lHWm54TU1ldGYzNS1jLWtQRjRHa1FoY3JUMkE4X0dkTmpDV204aWpmUlhVZmFKczZXRGllTE5aWnhPX2xwSE9tWmpzQmlXOVh6dTd2TnJJbWhaSmkyZHdrTzlxT2J3NmpkWmNBZHlzdUpmblVBd1JJS0ZSQlJKa3dqMlZ3cHBNZlozTFoxZ2tMLXB3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNQm1BZVJCYjVZajJsTEtXeFFXVU93Y2NpQ1cwbWhiN3l5d2tpNERrdF9vVUUwV0t2cE92dnd2NVJQRzZyN2xsVEQ5emtpNXlBNTNMX1B6cnAzM3F1bndYNTZfY0s2T3JmSGdYTHlDRmx3WnNhbWc4Yl90ek5rcmpqbW1NQWJ4WTF1aS1INU1HMjJpZF9aRGpsTkQxRUVTNVZUV0hBc2NmeVpOZnJjM3h3ZkM1Z2hEaldEWW5vTVdYNHhtZDVVZFp4Vm9KUzhaSzV2bWpMek5TMkZiNURnbzE3SlNRWnMxWW9kaUF3?oc=5</t>
         </is>
       </c>
       <c r="N100" s="2" t="inlineStr">
         <is>
-          <t>The News Mill</t>
+          <t>City and County of Honolulu (.gov)</t>
         </is>
       </c>
       <c r="O100" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-16 16:56:17</t>
-        </is>
-      </c>
-      <c r="B101" s="2" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="C101" s="2" t="inlineStr">
-        <is>
-          <t>Realty Income</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>City urges residents to stay safe as Hurricane Lala passes O‘ahu; TheBus service temporarily suspended due to extreme weather</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>颶風拉拉經過歐胡島時，市政府敦促居民保持安全；巴士服務因極端天氣而暫停</t>
-        </is>
-      </c>
-      <c r="F101" s="2" t="n">
-        <v>-0.917</v>
-      </c>
-      <c r="G101" s="2" t="inlineStr">
-        <is>
-          <t>OPERATIONS</t>
-        </is>
-      </c>
-      <c r="H101" s="2" t="inlineStr">
-        <is>
-          <t>NATURAL_DISASTER</t>
-        </is>
-      </c>
-      <c r="I101" s="2" t="inlineStr">
-        <is>
-          <t>天災</t>
-        </is>
-      </c>
-      <c r="J101" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K101" s="2" t="inlineStr">
-        <is>
-          <t>僅紀錄</t>
-        </is>
-      </c>
-      <c r="L101" s="2" t="inlineStr">
-        <is>
-          <t>hurricane</t>
-        </is>
-      </c>
-      <c r="M101" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNQm1BZVJCYjVZajJsTEtXeFFXVU93Y2NpQ1cwbWhiN3l5d2tpNERrdF9vVUUwV0t2cE92dnd2NVJQRzZyN2xsVEQ5emtpNXlBNTNMX1B6cnAzM3F1bndYNTZfY0s2T3JmSGdYTHlDRmx3WnNhbWc4Yl90ek5rcmpqbW1NQWJ4WTF1aS1INU1HMjJpZF9aRGpsTkQxRUVTNVZUV0hBc2NmeVpOZnJjM3h3ZkM1Z2hEaldEWW5vTVdYNHhtZDVVZFp4Vm9KUzhaSzV2bWpMek5TMkZiNURnbzE3SlNRWnMxWW9kaUF3?oc=5</t>
-        </is>
-      </c>
-      <c r="N101" s="2" t="inlineStr">
-        <is>
-          <t>City and County of Honolulu (.gov)</t>
-        </is>
-      </c>
-      <c r="O101" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O101"/>
+  <autoFilter ref="A1:O100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>